<commit_message>
feat(marine): add per-shipment minimum premium and correct stamp duty
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NgpxpZhjUPvBcqNwrsXRvp
</commit_message>
<xml_diff>
--- a/templates/quotation/quotation template.xlsx
+++ b/templates/quotation/quotation template.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9FB638-F80C-4357-A3F1-31C91A08BB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B54369-2263-4341-BF7E-49757DDFB820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="335">
   <si>
     <t>INSURED</t>
   </si>
@@ -1683,9 +1683,6 @@
     <t>{{bond_itl}}</t>
   </si>
   <si>
-    <t>{{bond_stamp_duty}}</t>
-  </si>
-  <si>
     <t>{{bond_total_premium}}</t>
   </si>
   <si>
@@ -1747,9 +1744,6 @@
     <t>{{guarantee_itl}}</t>
   </si>
   <si>
-    <t>{{guarantee_stamp_duty}}</t>
-  </si>
-  <si>
     <t>{{guarantee_total_premium}}</t>
   </si>
   <si>
@@ -1805,9 +1799,6 @@
     <t>{{custom_bond_itl}}</t>
   </si>
   <si>
-    <t>{{custom_bond_stamp_duty}}</t>
-  </si>
-  <si>
     <t>{{custom_bond_total_premium}}</t>
   </si>
   <si>
@@ -1910,6 +1901,86 @@
   </si>
   <si>
     <t>{{git_basic_premium}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>FROM {{marine_origin}} TO {{marine_destination}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>Incidental Loading (10%)</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> {{marine_incidental_loading}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Basic Sum Insured </t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> {{marine_basic_sum_insured}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>{{marine_rate}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>{{marine_line_premium}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>{{marine_total_basic_sum_insured}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>M Members          {{medical_m_count}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>M+1 Members      {{medical_m1_count}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>M+2 Members      {{medical_m2_count}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>M+3 Members      {{medical_m3_count}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>M+4 Members      {{medical_m4_count}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>{{medical_employee_count}} Employees</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>M+5 Members      {{medical_m5_count}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>{{el_any_one_person}}</t>
+  </si>
+  <si>
+    <t>{{el_any_one_occurrence}}</t>
+  </si>
+  <si>
+    <t>{{el_any_one_year}}</t>
+  </si>
+  <si>
+    <t>{{el_rate_percent}}%</t>
+  </si>
+  <si>
+    <t>{{marine_minimum_premium_label}}</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>{{marine_minimum_premium_amount}}</t>
     <phoneticPr fontId="10" type="noConversion"/>
   </si>
   <si>
@@ -1935,8 +2006,6 @@
 Institute classification cluase
 Institute replacement clause
 Institute radioactive contamination exclusion exclusion
-Institute standard conditions for cargo contracts
-Excluding unexplained losses
 Excluding caking and rainwater damage
 Excluding contamination other than by sea water
 Excluding spontaneous combustion, sweating, heating, spillage and hook dmage
@@ -1945,16 +2014,11 @@
 Excluding scratching,denting
 Political risks exclusion clause
 Excluding mechanical failure of refrigirators other than from a result of insured peril
-General average and salvage charges clause
 Packing Warranty
-Minimum premium: ksh. 5,000
 Loss due to delays (deterioration of stock) other than from as a result of insured perils is excluded
-Five Powers War Exclusion
-Seepage and Pollution Exclusion
 Specified territory Exclusion – Russia, Ukraine and Belarus Waters
 Excluding Hull War, Piracy, Terrorism and Related Perils
-Excluding water damage other than by sea water
-Sanction Clause
+Minimum premium: ksh. 5,000
 </t>
     </r>
     <r>
@@ -1978,66 +2042,6 @@
       <t xml:space="preserve">
 10% of consignment value minimum Kshs 50,000/-</t>
     </r>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>FROM {{marine_origin}} TO {{marine_destination}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>Incidental Loading (10%)</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> {{marine_incidental_loading}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Basic Sum Insured </t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve"> {{marine_basic_sum_insured}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{marine_rate}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{marine_line_premium}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{marine_total_basic_sum_insured}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>M Members          {{medical_m_count}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>M+1 Members      {{medical_m1_count}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>M+2 Members      {{medical_m2_count}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>M+3 Members      {{medical_m3_count}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>M+4 Members      {{medical_m4_count}}</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{medical_employee_count}} Employees</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
-    <t>M+5 Members      {{medical_m5_count}}</t>
     <phoneticPr fontId="10" type="noConversion"/>
   </si>
 </sst>
@@ -2272,7 +2276,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -2444,7 +2448,13 @@
     <xf numFmtId="43" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2482,27 +2492,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf applyNumberFormat="1" numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyNumberFormat="1" numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2957,12 +2946,12 @@
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="71"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="73"/>
     </row>
     <row r="3" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
@@ -2995,7 +2984,7 @@
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
       <c r="D5" s="11"/>
-      <c r="E5" s="61" t="s">
+      <c r="E5" s="63" t="s">
         <v>8</v>
       </c>
     </row>
@@ -3004,7 +2993,7 @@
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="13"/>
-      <c r="E6" s="61"/>
+      <c r="E6" s="63"/>
     </row>
     <row r="7" spans="1:5" ht="15.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
@@ -3013,7 +3002,7 @@
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="13"/>
-      <c r="E7" s="61"/>
+      <c r="E7" s="63"/>
     </row>
     <row r="8" spans="1:5" ht="88" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="15" t="s">
@@ -3022,7 +3011,7 @@
       <c r="B8" s="16"/>
       <c r="C8" s="10"/>
       <c r="D8" s="13"/>
-      <c r="E8" s="61"/>
+      <c r="E8" s="63"/>
     </row>
     <row r="9" spans="1:5" ht="15.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
@@ -3031,13 +3020,13 @@
       <c r="B9" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="73" t="s">
+      <c r="C9" s="59" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="61"/>
+      <c r="E9" s="63"/>
     </row>
     <row r="10" spans="1:5" ht="15.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
@@ -3046,7 +3035,7 @@
       <c r="B10" s="19"/>
       <c r="C10" s="20"/>
       <c r="D10" s="13"/>
-      <c r="E10" s="61"/>
+      <c r="E10" s="63"/>
     </row>
     <row r="11" spans="1:5" ht="15.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
@@ -3055,14 +3044,14 @@
       <c r="B11" s="19"/>
       <c r="C11" s="18"/>
       <c r="D11" s="13"/>
-      <c r="E11" s="61"/>
+      <c r="E11" s="63"/>
     </row>
     <row r="12" spans="1:5" ht="15.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="21"/>
       <c r="B12" s="17"/>
       <c r="C12" s="20"/>
       <c r="D12" s="13"/>
-      <c r="E12" s="61"/>
+      <c r="E12" s="63"/>
     </row>
     <row r="13" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
@@ -3071,7 +3060,7 @@
       <c r="B13" s="19"/>
       <c r="C13" s="18"/>
       <c r="D13" s="13"/>
-      <c r="E13" s="61"/>
+      <c r="E13" s="63"/>
     </row>
     <row r="14" spans="1:5" ht="15.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
@@ -3080,27 +3069,27 @@
       <c r="B14" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="73" t="s">
+      <c r="C14" s="59" t="s">
         <v>20</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="61"/>
+      <c r="E14" s="63"/>
     </row>
     <row r="15" spans="1:5" ht="15.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="23"/>
       <c r="B15" s="24"/>
       <c r="C15" s="18"/>
       <c r="D15" s="13"/>
-      <c r="E15" s="61"/>
+      <c r="E15" s="63"/>
     </row>
     <row r="16" spans="1:5" ht="15.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10"/>
       <c r="B16" s="17"/>
       <c r="C16" s="20"/>
       <c r="D16" s="13"/>
-      <c r="E16" s="61"/>
+      <c r="E16" s="63"/>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
@@ -3109,14 +3098,14 @@
       <c r="B17" s="19"/>
       <c r="C17" s="18"/>
       <c r="D17" s="13"/>
-      <c r="E17" s="61"/>
+      <c r="E17" s="63"/>
     </row>
     <row r="18" spans="1:5" ht="15.55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="9"/>
       <c r="B18" s="19"/>
       <c r="C18" s="18"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="61"/>
+      <c r="E18" s="63"/>
     </row>
     <row r="19" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
@@ -3125,7 +3114,7 @@
       <c r="B19" s="17"/>
       <c r="C19" s="18"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="61"/>
+      <c r="E19" s="63"/>
     </row>
     <row r="20" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
@@ -3136,7 +3125,7 @@
       </c>
       <c r="C20" s="25"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="61"/>
+      <c r="E20" s="63"/>
     </row>
     <row r="21" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
@@ -3147,7 +3136,7 @@
       </c>
       <c r="C21" s="18"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="61"/>
+      <c r="E21" s="63"/>
     </row>
     <row r="22" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
@@ -3156,84 +3145,84 @@
       <c r="B22" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="75" t="s">
+      <c r="C22" s="60" t="s">
         <v>30</v>
       </c>
       <c r="D22" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="61"/>
+      <c r="E22" s="63"/>
     </row>
     <row r="23" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="10"/>
       <c r="B23" s="17"/>
       <c r="C23" s="25"/>
       <c r="D23" s="13"/>
-      <c r="E23" s="61"/>
+      <c r="E23" s="63"/>
     </row>
     <row r="24" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
+        <v>289</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>290</v>
+      </c>
+      <c r="C24" s="60" t="s">
+        <v>291</v>
+      </c>
+      <c r="D24" s="13" t="s">
         <v>292</v>
       </c>
-      <c r="B24" s="17" t="s">
-        <v>293</v>
-      </c>
-      <c r="C24" s="75" t="s">
-        <v>294</v>
-      </c>
-      <c r="D24" s="13" t="s">
-        <v>295</v>
-      </c>
-      <c r="E24" s="61"/>
+      <c r="E24" s="63"/>
     </row>
     <row r="25" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="10"/>
       <c r="B25" s="17"/>
       <c r="C25" s="25"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="61"/>
+      <c r="E25" s="63"/>
     </row>
     <row r="26" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="10"/>
       <c r="B26" s="17"/>
       <c r="C26" s="25"/>
       <c r="D26" s="13"/>
-      <c r="E26" s="61"/>
+      <c r="E26" s="63"/>
     </row>
     <row r="27" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10"/>
       <c r="B27" s="17"/>
       <c r="C27" s="25"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="61"/>
+      <c r="E27" s="63"/>
     </row>
     <row r="28" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="10"/>
       <c r="B28" s="17"/>
       <c r="C28" s="25"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="61"/>
+      <c r="E28" s="63"/>
     </row>
     <row r="29" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="10"/>
       <c r="B29" s="17"/>
       <c r="C29" s="25"/>
       <c r="D29" s="13"/>
-      <c r="E29" s="61"/>
+      <c r="E29" s="63"/>
     </row>
     <row r="30" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="21"/>
       <c r="B30" s="17"/>
       <c r="C30" s="20"/>
       <c r="D30" s="13"/>
-      <c r="E30" s="61"/>
+      <c r="E30" s="63"/>
     </row>
     <row r="31" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
       <c r="D31" s="13"/>
-      <c r="E31" s="61"/>
+      <c r="E31" s="63"/>
     </row>
     <row r="32" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="10"/>
@@ -3244,7 +3233,7 @@
       <c r="D32" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="E32" s="61"/>
+      <c r="E32" s="63"/>
     </row>
     <row r="33" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="10"/>
@@ -3257,7 +3246,7 @@
       <c r="D33" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="E33" s="61"/>
+      <c r="E33" s="63"/>
     </row>
     <row r="34" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="10"/>
@@ -3270,7 +3259,7 @@
       <c r="D34" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="E34" s="61"/>
+      <c r="E34" s="63"/>
     </row>
     <row r="35" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10"/>
@@ -3281,7 +3270,7 @@
       <c r="D35" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="E35" s="61"/>
+      <c r="E35" s="63"/>
     </row>
     <row r="36" spans="1:5" ht="36.549999999999997" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="28"/>
@@ -3292,7 +3281,7 @@
       <c r="D36" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="E36" s="62"/>
+      <c r="E36" s="64"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="7"/>
@@ -3308,7 +3297,7 @@
       <c r="B38" s="10"/>
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
-      <c r="E38" s="61" t="s">
+      <c r="E38" s="63" t="s">
         <v>43</v>
       </c>
     </row>
@@ -3317,7 +3306,7 @@
       <c r="B39" s="10"/>
       <c r="C39" s="10"/>
       <c r="D39" s="13"/>
-      <c r="E39" s="61"/>
+      <c r="E39" s="63"/>
     </row>
     <row r="40" spans="1:5" ht="46.3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="14" t="s">
@@ -3326,7 +3315,7 @@
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
       <c r="D40" s="13"/>
-      <c r="E40" s="61"/>
+      <c r="E40" s="63"/>
     </row>
     <row r="41" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
@@ -3335,14 +3324,14 @@
       <c r="B41" s="10"/>
       <c r="C41" s="10"/>
       <c r="D41" s="13"/>
-      <c r="E41" s="61"/>
+      <c r="E41" s="63"/>
     </row>
     <row r="42" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="10"/>
       <c r="B42" s="17"/>
       <c r="C42" s="18"/>
       <c r="D42" s="13"/>
-      <c r="E42" s="61"/>
+      <c r="E42" s="63"/>
     </row>
     <row r="43" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
@@ -3353,119 +3342,119 @@
       </c>
       <c r="C43" s="18"/>
       <c r="D43" s="13"/>
-      <c r="E43" s="61"/>
+      <c r="E43" s="63"/>
     </row>
     <row r="44" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="10"/>
       <c r="B44" s="17"/>
       <c r="C44" s="18"/>
       <c r="D44" s="13"/>
-      <c r="E44" s="61"/>
+      <c r="E44" s="63"/>
     </row>
     <row r="45" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="10"/>
       <c r="B45" s="17"/>
       <c r="C45" s="18"/>
       <c r="D45" s="13"/>
-      <c r="E45" s="61"/>
+      <c r="E45" s="63"/>
     </row>
     <row r="46" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="10"/>
       <c r="B46" s="17"/>
       <c r="C46" s="18"/>
       <c r="D46" s="13"/>
-      <c r="E46" s="61"/>
+      <c r="E46" s="63"/>
     </row>
     <row r="47" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10"/>
       <c r="B47" s="17"/>
       <c r="C47" s="18"/>
       <c r="D47" s="13"/>
-      <c r="E47" s="61"/>
+      <c r="E47" s="63"/>
     </row>
     <row r="48" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="10"/>
       <c r="B48" s="17"/>
       <c r="C48" s="18"/>
       <c r="D48" s="13"/>
-      <c r="E48" s="61"/>
+      <c r="E48" s="63"/>
     </row>
     <row r="49" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="10"/>
       <c r="B49" s="17"/>
       <c r="C49" s="18"/>
       <c r="D49" s="13"/>
-      <c r="E49" s="61"/>
+      <c r="E49" s="63"/>
     </row>
     <row r="50" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="10"/>
       <c r="B50" s="17"/>
       <c r="C50" s="18"/>
       <c r="D50" s="13"/>
-      <c r="E50" s="61"/>
+      <c r="E50" s="63"/>
     </row>
     <row r="51" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10"/>
       <c r="B51" s="17"/>
       <c r="C51" s="18"/>
       <c r="D51" s="13"/>
-      <c r="E51" s="61"/>
+      <c r="E51" s="63"/>
     </row>
     <row r="52" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="10"/>
       <c r="B52" s="17"/>
       <c r="C52" s="18"/>
       <c r="D52" s="13"/>
-      <c r="E52" s="61"/>
+      <c r="E52" s="63"/>
     </row>
     <row r="53" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="10"/>
       <c r="B53" s="17"/>
       <c r="C53" s="18"/>
       <c r="D53" s="13"/>
-      <c r="E53" s="61"/>
+      <c r="E53" s="63"/>
     </row>
     <row r="54" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="10"/>
       <c r="B54" s="17"/>
       <c r="C54" s="18"/>
       <c r="D54" s="13"/>
-      <c r="E54" s="61"/>
+      <c r="E54" s="63"/>
     </row>
     <row r="55" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="10"/>
       <c r="B55" s="17"/>
       <c r="C55" s="18"/>
       <c r="D55" s="13"/>
-      <c r="E55" s="61"/>
+      <c r="E55" s="63"/>
     </row>
     <row r="56" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="10"/>
       <c r="B56" s="17"/>
       <c r="C56" s="18"/>
       <c r="D56" s="13"/>
-      <c r="E56" s="61"/>
+      <c r="E56" s="63"/>
     </row>
     <row r="57" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="10"/>
       <c r="B57" s="17"/>
       <c r="C57" s="18"/>
       <c r="D57" s="13"/>
-      <c r="E57" s="61"/>
+      <c r="E57" s="63"/>
     </row>
     <row r="58" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="10"/>
       <c r="B58" s="17"/>
       <c r="C58" s="18"/>
       <c r="D58" s="13"/>
-      <c r="E58" s="61"/>
+      <c r="E58" s="63"/>
     </row>
     <row r="59" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="10"/>
       <c r="B59" s="17"/>
       <c r="C59" s="18"/>
       <c r="D59" s="13"/>
-      <c r="E59" s="61"/>
+      <c r="E59" s="63"/>
     </row>
     <row r="60" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="21" t="s">
@@ -3474,20 +3463,20 @@
       <c r="B60" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="C60" s="73" t="s">
+      <c r="C60" s="59" t="s">
         <v>50</v>
       </c>
       <c r="D60" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="E60" s="61"/>
+      <c r="E60" s="63"/>
     </row>
     <row r="61" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="10"/>
       <c r="B61" s="23"/>
       <c r="C61" s="10"/>
       <c r="D61" s="13"/>
-      <c r="E61" s="61"/>
+      <c r="E61" s="63"/>
     </row>
     <row r="62" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="10"/>
@@ -3498,7 +3487,7 @@
       <c r="D62" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="E62" s="61"/>
+      <c r="E62" s="63"/>
     </row>
     <row r="63" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="10"/>
@@ -3511,7 +3500,7 @@
       <c r="D63" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="E63" s="61"/>
+      <c r="E63" s="63"/>
     </row>
     <row r="64" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="10"/>
@@ -3524,7 +3513,7 @@
       <c r="D64" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="E64" s="61"/>
+      <c r="E64" s="63"/>
     </row>
     <row r="65" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="10"/>
@@ -3535,7 +3524,7 @@
       <c r="D65" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="E65" s="61"/>
+      <c r="E65" s="63"/>
     </row>
     <row r="66" spans="1:5" ht="36.549999999999997" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="28"/>
@@ -3546,7 +3535,7 @@
       <c r="D66" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="E66" s="62"/>
+      <c r="E66" s="64"/>
     </row>
     <row r="67" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="31"/>
@@ -3562,7 +3551,7 @@
       <c r="B68" s="10"/>
       <c r="C68" s="10"/>
       <c r="D68" s="13"/>
-      <c r="E68" s="61" t="s">
+      <c r="E68" s="63" t="s">
         <v>57</v>
       </c>
     </row>
@@ -3571,53 +3560,47 @@
       <c r="B69" s="10"/>
       <c r="C69" s="10"/>
       <c r="D69" s="13"/>
-      <c r="E69" s="61"/>
+      <c r="E69" s="63"/>
     </row>
     <row r="70" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B70" s="13" t="inlineStr">
-        <is>
-          <t>{{el_any_one_person}}</t>
-        </is>
+      <c r="B70" s="13" t="s">
+        <v>328</v>
       </c>
       <c r="C70" s="10"/>
       <c r="D70" s="13"/>
-      <c r="E70" s="61"/>
+      <c r="E70" s="63"/>
     </row>
     <row r="71" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B71" s="13" t="inlineStr">
-        <is>
-          <t>{{el_any_one_occurrence}}</t>
-        </is>
+      <c r="B71" s="13" t="s">
+        <v>329</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="13"/>
-      <c r="E71" s="61"/>
+      <c r="E71" s="63"/>
     </row>
     <row r="72" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B72" s="13" t="inlineStr">
-        <is>
-          <t>{{el_any_one_year}}</t>
-        </is>
+      <c r="B72" s="13" t="s">
+        <v>330</v>
       </c>
       <c r="C72" s="10"/>
       <c r="D72" s="13"/>
-      <c r="E72" s="61"/>
+      <c r="E72" s="63"/>
     </row>
     <row r="73" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="10"/>
       <c r="B73" s="10"/>
       <c r="C73" s="10"/>
       <c r="D73" s="33"/>
-      <c r="E73" s="61"/>
+      <c r="E73" s="63"/>
     </row>
     <row r="74" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="9" t="s">
@@ -3627,22 +3610,20 @@
         <f>D62</f>
         <v>{{wiba_gross_premium}}</v>
       </c>
-      <c r="C74" s="34" t="inlineStr">
-        <is>
-          <t>{{el_rate_percent}}%</t>
-        </is>
+      <c r="C74" s="34" t="s">
+        <v>331</v>
       </c>
       <c r="D74" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="E74" s="61"/>
+      <c r="E74" s="63"/>
     </row>
     <row r="75" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="10"/>
       <c r="B75" s="10"/>
       <c r="C75" s="10"/>
       <c r="D75" s="13"/>
-      <c r="E75" s="61"/>
+      <c r="E75" s="63"/>
     </row>
     <row r="76" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="21"/>
@@ -3654,7 +3635,7 @@
         <f>D74</f>
         <v xml:space="preserve"> {{el_gross_premium}}</v>
       </c>
-      <c r="E76" s="61"/>
+      <c r="E76" s="63"/>
     </row>
     <row r="77" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="10"/>
@@ -3667,7 +3648,7 @@
       <c r="D77" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="E77" s="61"/>
+      <c r="E77" s="63"/>
     </row>
     <row r="78" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="10"/>
@@ -3680,7 +3661,7 @@
       <c r="D78" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E78" s="61"/>
+      <c r="E78" s="63"/>
     </row>
     <row r="79" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="10"/>
@@ -3691,7 +3672,7 @@
       <c r="D79" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="E79" s="61"/>
+      <c r="E79" s="63"/>
     </row>
     <row r="80" spans="1:5" ht="36.549999999999997" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="28"/>
@@ -3702,7 +3683,7 @@
       <c r="D80" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="E80" s="62"/>
+      <c r="E80" s="64"/>
     </row>
     <row r="81" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="10"/>
@@ -3718,7 +3699,7 @@
       <c r="B82" s="10"/>
       <c r="C82" s="10"/>
       <c r="D82" s="13"/>
-      <c r="E82" s="61" t="s">
+      <c r="E82" s="63" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3727,118 +3708,118 @@
       <c r="B83" s="10"/>
       <c r="C83" s="10"/>
       <c r="D83" s="13"/>
-      <c r="E83" s="61"/>
+      <c r="E83" s="63"/>
     </row>
     <row r="84" spans="1:5" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="10" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B84" s="36" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C84" s="10"/>
       <c r="D84" s="13"/>
-      <c r="E84" s="61"/>
+      <c r="E84" s="63"/>
     </row>
     <row r="85" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="10"/>
       <c r="B85" s="36"/>
       <c r="C85" s="10"/>
       <c r="D85" s="13"/>
-      <c r="E85" s="61"/>
+      <c r="E85" s="63"/>
     </row>
     <row r="86" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="10" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B86" s="36" t="s">
-        <v>313</v>
-      </c>
-      <c r="C86" s="72" t="s">
-        <v>299</v>
+        <v>310</v>
+      </c>
+      <c r="C86" s="59" t="s">
+        <v>296</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>300</v>
-      </c>
-      <c r="E86" s="61"/>
+        <v>297</v>
+      </c>
+      <c r="E86" s="63"/>
     </row>
     <row r="87" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="10"/>
       <c r="B87" s="36"/>
       <c r="C87" s="10"/>
       <c r="D87" s="13"/>
-      <c r="E87" s="61"/>
+      <c r="E87" s="63"/>
     </row>
     <row r="88" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="10" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B88" s="36" t="s">
-        <v>296</v>
-      </c>
-      <c r="C88" s="72" t="s">
-        <v>297</v>
+        <v>293</v>
+      </c>
+      <c r="C88" s="59" t="s">
+        <v>294</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>301</v>
-      </c>
-      <c r="E88" s="61"/>
+        <v>298</v>
+      </c>
+      <c r="E88" s="63"/>
     </row>
     <row r="89" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="10"/>
       <c r="B89" s="36"/>
       <c r="C89" s="10"/>
       <c r="D89" s="13"/>
-      <c r="E89" s="61"/>
+      <c r="E89" s="63"/>
     </row>
     <row r="90" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="10"/>
       <c r="B90" s="36"/>
       <c r="C90" s="10"/>
       <c r="D90" s="13"/>
-      <c r="E90" s="61"/>
+      <c r="E90" s="63"/>
     </row>
     <row r="91" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="10"/>
       <c r="B91" s="36"/>
       <c r="C91" s="20"/>
       <c r="D91" s="13"/>
-      <c r="E91" s="61"/>
+      <c r="E91" s="63"/>
     </row>
     <row r="92" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="10"/>
       <c r="B92" s="36"/>
       <c r="C92" s="20"/>
       <c r="D92" s="13"/>
-      <c r="E92" s="61"/>
+      <c r="E92" s="63"/>
     </row>
     <row r="93" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="10"/>
       <c r="B93" s="36"/>
       <c r="C93" s="20"/>
       <c r="D93" s="13"/>
-      <c r="E93" s="61"/>
+      <c r="E93" s="63"/>
     </row>
     <row r="94" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="10"/>
       <c r="B94" s="17"/>
       <c r="C94" s="20"/>
       <c r="D94" s="13"/>
-      <c r="E94" s="61"/>
+      <c r="E94" s="63"/>
     </row>
     <row r="95" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="21"/>
       <c r="B95" s="17"/>
       <c r="C95" s="20"/>
       <c r="D95" s="13"/>
-      <c r="E95" s="61"/>
+      <c r="E95" s="63"/>
     </row>
     <row r="96" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="10"/>
       <c r="B96" s="21"/>
       <c r="C96" s="34"/>
       <c r="D96" s="13"/>
-      <c r="E96" s="61"/>
+      <c r="E96" s="63"/>
     </row>
     <row r="97" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="21"/>
@@ -3849,7 +3830,7 @@
       <c r="D97" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="E97" s="61"/>
+      <c r="E97" s="63"/>
     </row>
     <row r="98" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="10"/>
@@ -3862,7 +3843,7 @@
       <c r="D98" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="E98" s="61"/>
+      <c r="E98" s="63"/>
     </row>
     <row r="99" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="10"/>
@@ -3875,7 +3856,7 @@
       <c r="D99" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="E99" s="61"/>
+      <c r="E99" s="63"/>
     </row>
     <row r="100" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="10"/>
@@ -3886,14 +3867,14 @@
       <c r="D100" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E100" s="61"/>
+      <c r="E100" s="63"/>
     </row>
     <row r="101" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="10"/>
       <c r="B101" s="9"/>
       <c r="C101" s="10"/>
       <c r="D101" s="13"/>
-      <c r="E101" s="61"/>
+      <c r="E101" s="63"/>
     </row>
     <row r="102" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="28"/>
@@ -3904,7 +3885,7 @@
       <c r="D102" s="30" t="s">
         <v>72</v>
       </c>
-      <c r="E102" s="62"/>
+      <c r="E102" s="64"/>
     </row>
     <row r="103" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="10"/>
@@ -3919,7 +3900,7 @@
       <c r="B104" s="10"/>
       <c r="C104" s="10"/>
       <c r="D104" s="13"/>
-      <c r="E104" s="61" t="s">
+      <c r="E104" s="63" t="s">
         <v>74</v>
       </c>
     </row>
@@ -3928,7 +3909,7 @@
       <c r="B105" s="10"/>
       <c r="C105" s="10"/>
       <c r="D105" s="13"/>
-      <c r="E105" s="61"/>
+      <c r="E105" s="63"/>
     </row>
     <row r="106" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="10" t="s">
@@ -3939,14 +3920,14 @@
       </c>
       <c r="C106" s="10"/>
       <c r="D106" s="13"/>
-      <c r="E106" s="61"/>
+      <c r="E106" s="63"/>
     </row>
     <row r="107" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="10"/>
       <c r="B107" s="13"/>
       <c r="C107" s="10"/>
       <c r="D107" s="13"/>
-      <c r="E107" s="61"/>
+      <c r="E107" s="63"/>
     </row>
     <row r="108" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="10" t="s">
@@ -3957,14 +3938,14 @@
       </c>
       <c r="C108" s="10"/>
       <c r="D108" s="13"/>
-      <c r="E108" s="61"/>
+      <c r="E108" s="63"/>
     </row>
     <row r="109" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="10"/>
       <c r="B109" s="13"/>
       <c r="C109" s="10"/>
       <c r="D109" s="13"/>
-      <c r="E109" s="61"/>
+      <c r="E109" s="63"/>
     </row>
     <row r="110" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="10" t="s">
@@ -3973,69 +3954,69 @@
       <c r="B110" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="C110" s="73" t="s">
+      <c r="C110" s="59" t="s">
         <v>78</v>
       </c>
       <c r="D110" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="E110" s="61"/>
+      <c r="E110" s="63"/>
     </row>
     <row r="111" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="10"/>
       <c r="B111" s="10"/>
       <c r="C111" s="10"/>
       <c r="D111" s="13"/>
-      <c r="E111" s="61"/>
+      <c r="E111" s="63"/>
     </row>
     <row r="112" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A112" s="10"/>
       <c r="B112" s="10"/>
       <c r="C112" s="10"/>
       <c r="D112" s="13"/>
-      <c r="E112" s="61"/>
+      <c r="E112" s="63"/>
     </row>
     <row r="113" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" s="10"/>
       <c r="B113" s="10"/>
       <c r="C113" s="10"/>
       <c r="D113" s="13"/>
-      <c r="E113" s="61"/>
+      <c r="E113" s="63"/>
     </row>
     <row r="114" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="10"/>
       <c r="B114" s="10"/>
       <c r="C114" s="10"/>
       <c r="D114" s="13"/>
-      <c r="E114" s="61"/>
+      <c r="E114" s="63"/>
     </row>
     <row r="115" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115" s="10"/>
       <c r="B115" s="10"/>
       <c r="C115" s="10"/>
       <c r="D115" s="13"/>
-      <c r="E115" s="61"/>
+      <c r="E115" s="63"/>
     </row>
     <row r="116" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A116" s="10"/>
       <c r="B116" s="10"/>
       <c r="C116" s="10"/>
       <c r="D116" s="13"/>
-      <c r="E116" s="61"/>
+      <c r="E116" s="63"/>
     </row>
     <row r="117" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" s="9"/>
       <c r="B117" s="17"/>
       <c r="C117" s="34"/>
       <c r="D117" s="13"/>
-      <c r="E117" s="61"/>
+      <c r="E117" s="63"/>
     </row>
     <row r="118" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" s="10"/>
       <c r="B118" s="10"/>
       <c r="C118" s="10"/>
       <c r="D118" s="13"/>
-      <c r="E118" s="61"/>
+      <c r="E118" s="63"/>
     </row>
     <row r="119" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="21"/>
@@ -4046,7 +4027,7 @@
       <c r="D119" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="E119" s="61"/>
+      <c r="E119" s="63"/>
     </row>
     <row r="120" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" s="10"/>
@@ -4059,7 +4040,7 @@
       <c r="D120" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="E120" s="61"/>
+      <c r="E120" s="63"/>
     </row>
     <row r="121" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" s="10"/>
@@ -4072,7 +4053,7 @@
       <c r="D121" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="E121" s="61"/>
+      <c r="E121" s="63"/>
     </row>
     <row r="122" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" s="10"/>
@@ -4083,14 +4064,14 @@
       <c r="D122" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="E122" s="61"/>
+      <c r="E122" s="63"/>
     </row>
     <row r="123" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="10"/>
       <c r="B123" s="9"/>
       <c r="C123" s="10"/>
       <c r="D123" s="13"/>
-      <c r="E123" s="61"/>
+      <c r="E123" s="63"/>
     </row>
     <row r="124" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="28"/>
@@ -4101,7 +4082,7 @@
       <c r="D124" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="E124" s="62"/>
+      <c r="E124" s="64"/>
     </row>
     <row r="125" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A125" s="10"/>
@@ -4123,7 +4104,7 @@
       <c r="B127" s="10"/>
       <c r="C127" s="10"/>
       <c r="D127" s="11"/>
-      <c r="E127" s="61" t="s">
+      <c r="E127" s="63" t="s">
         <v>85</v>
       </c>
     </row>
@@ -4132,7 +4113,7 @@
       <c r="B128" s="10"/>
       <c r="C128" s="10"/>
       <c r="D128" s="11"/>
-      <c r="E128" s="61"/>
+      <c r="E128" s="63"/>
     </row>
     <row r="129" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" s="10" t="s">
@@ -4143,7 +4124,7 @@
       </c>
       <c r="C129" s="18"/>
       <c r="D129" s="13"/>
-      <c r="E129" s="61"/>
+      <c r="E129" s="63"/>
     </row>
     <row r="130" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130" s="10" t="s">
@@ -4154,7 +4135,7 @@
       </c>
       <c r="C130" s="34"/>
       <c r="D130" s="13"/>
-      <c r="E130" s="61"/>
+      <c r="E130" s="63"/>
     </row>
     <row r="131" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" s="10" t="s">
@@ -4165,21 +4146,21 @@
       </c>
       <c r="C131" s="10"/>
       <c r="D131" s="13"/>
-      <c r="E131" s="61"/>
+      <c r="E131" s="63"/>
     </row>
     <row r="132" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" s="10"/>
       <c r="B132" s="38"/>
       <c r="C132" s="18"/>
       <c r="D132" s="13"/>
-      <c r="E132" s="61"/>
+      <c r="E132" s="63"/>
     </row>
     <row r="133" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A133" s="10"/>
       <c r="B133" s="38"/>
       <c r="C133" s="18"/>
       <c r="D133" s="13"/>
-      <c r="E133" s="61"/>
+      <c r="E133" s="63"/>
     </row>
     <row r="134" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A134" s="21" t="s">
@@ -4188,27 +4169,27 @@
       <c r="B134" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C134" s="74" t="s">
+      <c r="C134" s="59" t="s">
         <v>93</v>
       </c>
       <c r="D134" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="E134" s="61"/>
+      <c r="E134" s="63"/>
     </row>
     <row r="135" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A135" s="21"/>
       <c r="B135" s="19"/>
       <c r="C135" s="20"/>
       <c r="D135" s="13"/>
-      <c r="E135" s="61"/>
+      <c r="E135" s="63"/>
     </row>
     <row r="136" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A136" s="21"/>
       <c r="B136" s="17"/>
       <c r="C136" s="20"/>
       <c r="D136" s="13"/>
-      <c r="E136" s="61"/>
+      <c r="E136" s="63"/>
     </row>
     <row r="137" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A137" s="21"/>
@@ -4221,7 +4202,7 @@
       <c r="D137" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="E137" s="61"/>
+      <c r="E137" s="63"/>
     </row>
     <row r="138" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A138" s="21"/>
@@ -4234,43 +4215,43 @@
       <c r="D138" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="E138" s="61"/>
+      <c r="E138" s="63"/>
     </row>
     <row r="139" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A139" s="21"/>
       <c r="B139" s="19"/>
       <c r="C139" s="18"/>
       <c r="D139" s="13"/>
-      <c r="E139" s="61"/>
+      <c r="E139" s="63"/>
     </row>
     <row r="140" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140" s="21" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B140" s="19" t="s">
-        <v>302</v>
-      </c>
-      <c r="C140" s="73" t="s">
-        <v>303</v>
+        <v>299</v>
+      </c>
+      <c r="C140" s="59" t="s">
+        <v>300</v>
       </c>
       <c r="D140" s="13" t="s">
-        <v>304</v>
-      </c>
-      <c r="E140" s="61"/>
+        <v>301</v>
+      </c>
+      <c r="E140" s="63"/>
     </row>
     <row r="141" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A141" s="21"/>
       <c r="B141" s="17"/>
       <c r="C141" s="18"/>
       <c r="D141" s="13"/>
-      <c r="E141" s="61"/>
+      <c r="E141" s="63"/>
     </row>
     <row r="142" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A142" s="10"/>
       <c r="B142" s="10"/>
       <c r="C142" s="10"/>
       <c r="D142" s="13"/>
-      <c r="E142" s="61"/>
+      <c r="E142" s="63"/>
     </row>
     <row r="143" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A143" s="10"/>
@@ -4281,7 +4262,7 @@
       <c r="D143" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="E143" s="61"/>
+      <c r="E143" s="63"/>
     </row>
     <row r="144" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144" s="10"/>
@@ -4294,7 +4275,7 @@
       <c r="D144" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="E144" s="61"/>
+      <c r="E144" s="63"/>
     </row>
     <row r="145" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145" s="10"/>
@@ -4307,7 +4288,7 @@
       <c r="D145" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E145" s="61"/>
+      <c r="E145" s="63"/>
     </row>
     <row r="146" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146" s="10"/>
@@ -4318,7 +4299,7 @@
       <c r="D146" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="E146" s="61"/>
+      <c r="E146" s="63"/>
     </row>
     <row r="147" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A147" s="28"/>
@@ -4329,7 +4310,7 @@
       <c r="D147" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="E147" s="62"/>
+      <c r="E147" s="64"/>
     </row>
     <row r="148" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A148" s="10"/>
@@ -4344,7 +4325,7 @@
       <c r="B149" s="10"/>
       <c r="C149" s="10"/>
       <c r="D149" s="11"/>
-      <c r="E149" s="60" t="s">
+      <c r="E149" s="62" t="s">
         <v>105</v>
       </c>
     </row>
@@ -4353,7 +4334,7 @@
       <c r="B150" s="10"/>
       <c r="C150" s="10"/>
       <c r="D150" s="11"/>
-      <c r="E150" s="60"/>
+      <c r="E150" s="62"/>
     </row>
     <row r="151" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A151" s="10" t="s">
@@ -4364,7 +4345,7 @@
       </c>
       <c r="C151" s="10"/>
       <c r="D151" s="13"/>
-      <c r="E151" s="61"/>
+      <c r="E151" s="63"/>
     </row>
     <row r="152" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A152" s="10" t="s">
@@ -4375,21 +4356,21 @@
       </c>
       <c r="C152" s="10"/>
       <c r="D152" s="13"/>
-      <c r="E152" s="61"/>
+      <c r="E152" s="63"/>
     </row>
     <row r="153" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A153" s="10"/>
       <c r="B153" s="38"/>
       <c r="C153" s="10"/>
       <c r="D153" s="13"/>
-      <c r="E153" s="61"/>
+      <c r="E153" s="63"/>
     </row>
     <row r="154" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A154" s="10"/>
       <c r="B154" s="36"/>
       <c r="C154" s="18"/>
       <c r="D154" s="13"/>
-      <c r="E154" s="61"/>
+      <c r="E154" s="63"/>
     </row>
     <row r="155" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A155" s="21" t="s">
@@ -4398,11 +4379,11 @@
       <c r="B155" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="C155" s="74" t="s">
+      <c r="C155" s="59" t="s">
         <v>111</v>
       </c>
       <c r="D155" s="13"/>
-      <c r="E155" s="61"/>
+      <c r="E155" s="63"/>
     </row>
     <row r="156" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A156" s="21" t="s">
@@ -4411,34 +4392,34 @@
       <c r="B156" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="C156" s="74" t="s">
+      <c r="C156" s="59" t="s">
         <v>114</v>
       </c>
       <c r="D156" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="E156" s="61"/>
+      <c r="E156" s="63"/>
     </row>
     <row r="157" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A157" s="21"/>
       <c r="B157" s="17"/>
       <c r="C157" s="18"/>
       <c r="D157" s="13"/>
-      <c r="E157" s="61"/>
+      <c r="E157" s="63"/>
     </row>
     <row r="158" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A158" s="21"/>
       <c r="B158" s="17"/>
       <c r="C158" s="18"/>
       <c r="D158" s="13"/>
-      <c r="E158" s="61"/>
+      <c r="E158" s="63"/>
     </row>
     <row r="159" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A159" s="10"/>
       <c r="B159" s="10"/>
       <c r="C159" s="10"/>
       <c r="D159" s="13"/>
-      <c r="E159" s="61"/>
+      <c r="E159" s="63"/>
     </row>
     <row r="160" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A160" s="10"/>
@@ -4449,7 +4430,7 @@
       <c r="D160" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="E160" s="61"/>
+      <c r="E160" s="63"/>
     </row>
     <row r="161" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A161" s="10"/>
@@ -4462,7 +4443,7 @@
       <c r="D161" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="E161" s="61"/>
+      <c r="E161" s="63"/>
     </row>
     <row r="162" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A162" s="10"/>
@@ -4475,7 +4456,7 @@
       <c r="D162" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="E162" s="61"/>
+      <c r="E162" s="63"/>
     </row>
     <row r="163" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A163" s="10"/>
@@ -4486,7 +4467,7 @@
       <c r="D163" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="E163" s="61"/>
+      <c r="E163" s="63"/>
     </row>
     <row r="164" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A164" s="28"/>
@@ -4497,7 +4478,7 @@
       <c r="D164" s="30" t="s">
         <v>119</v>
       </c>
-      <c r="E164" s="62"/>
+      <c r="E164" s="64"/>
     </row>
     <row r="165" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A165" s="10"/>
@@ -4512,7 +4493,7 @@
       <c r="B166" s="10"/>
       <c r="C166" s="10"/>
       <c r="D166" s="11"/>
-      <c r="E166" s="61" t="s">
+      <c r="E166" s="63" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4521,7 +4502,7 @@
       <c r="B167" s="10"/>
       <c r="C167" s="10"/>
       <c r="D167" s="13"/>
-      <c r="E167" s="61"/>
+      <c r="E167" s="63"/>
     </row>
     <row r="168" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A168" s="14" t="s">
@@ -4530,7 +4511,7 @@
       <c r="B168" s="10"/>
       <c r="C168" s="10"/>
       <c r="D168" s="13"/>
-      <c r="E168" s="61"/>
+      <c r="E168" s="63"/>
     </row>
     <row r="169" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A169" s="15" t="s">
@@ -4539,63 +4520,63 @@
       <c r="B169" s="10"/>
       <c r="C169" s="10"/>
       <c r="D169" s="13"/>
-      <c r="E169" s="61"/>
+      <c r="E169" s="63"/>
     </row>
     <row r="170" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A170" s="15"/>
       <c r="B170" s="10"/>
       <c r="C170" s="10"/>
       <c r="D170" s="13"/>
-      <c r="E170" s="61"/>
+      <c r="E170" s="63"/>
     </row>
     <row r="171" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A171" s="15"/>
       <c r="B171" s="10"/>
       <c r="C171" s="10"/>
       <c r="D171" s="13"/>
-      <c r="E171" s="61"/>
+      <c r="E171" s="63"/>
     </row>
     <row r="172" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A172" s="15"/>
       <c r="B172" s="10"/>
       <c r="C172" s="10"/>
       <c r="D172" s="13"/>
-      <c r="E172" s="61"/>
+      <c r="E172" s="63"/>
     </row>
     <row r="173" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A173" s="15"/>
       <c r="B173" s="10"/>
       <c r="C173" s="10"/>
       <c r="D173" s="13"/>
-      <c r="E173" s="61"/>
+      <c r="E173" s="63"/>
     </row>
     <row r="174" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A174" s="15"/>
       <c r="B174" s="10"/>
       <c r="C174" s="10"/>
       <c r="D174" s="13"/>
-      <c r="E174" s="61"/>
+      <c r="E174" s="63"/>
     </row>
     <row r="175" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A175" s="15"/>
       <c r="B175" s="10"/>
       <c r="C175" s="10"/>
       <c r="D175" s="13"/>
-      <c r="E175" s="61"/>
+      <c r="E175" s="63"/>
     </row>
     <row r="176" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A176" s="15"/>
       <c r="B176" s="10"/>
       <c r="C176" s="10"/>
       <c r="D176" s="13"/>
-      <c r="E176" s="61"/>
+      <c r="E176" s="63"/>
     </row>
     <row r="177" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A177" s="10"/>
       <c r="B177" s="17"/>
       <c r="C177" s="18"/>
       <c r="D177" s="13"/>
-      <c r="E177" s="61"/>
+      <c r="E177" s="63"/>
     </row>
     <row r="178" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A178" s="23" t="s">
@@ -4604,56 +4585,56 @@
       <c r="B178" s="36" t="s">
         <v>125</v>
       </c>
-      <c r="C178" s="73" t="s">
+      <c r="C178" s="59" t="s">
         <v>126</v>
       </c>
       <c r="D178" s="13" t="s">
-        <v>315</v>
-      </c>
-      <c r="E178" s="61"/>
+        <v>312</v>
+      </c>
+      <c r="E178" s="63"/>
     </row>
     <row r="179" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A179" s="23"/>
       <c r="B179" s="36"/>
       <c r="C179" s="18"/>
       <c r="D179" s="13"/>
-      <c r="E179" s="61"/>
+      <c r="E179" s="63"/>
     </row>
     <row r="180" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A180" s="23" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B180" s="36" t="s">
-        <v>305</v>
-      </c>
-      <c r="C180" s="73" t="s">
-        <v>306</v>
+        <v>302</v>
+      </c>
+      <c r="C180" s="59" t="s">
+        <v>303</v>
       </c>
       <c r="D180" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="E180" s="61"/>
+        <v>304</v>
+      </c>
+      <c r="E180" s="63"/>
     </row>
     <row r="181" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A181" s="23"/>
       <c r="B181" s="36"/>
       <c r="C181" s="18"/>
       <c r="D181" s="13"/>
-      <c r="E181" s="61"/>
+      <c r="E181" s="63"/>
     </row>
     <row r="182" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A182" s="21"/>
       <c r="B182" s="17"/>
       <c r="C182" s="20"/>
       <c r="D182" s="13"/>
-      <c r="E182" s="61"/>
+      <c r="E182" s="63"/>
     </row>
     <row r="183" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A183" s="10"/>
       <c r="B183" s="10"/>
       <c r="C183" s="10"/>
       <c r="D183" s="13"/>
-      <c r="E183" s="61"/>
+      <c r="E183" s="63"/>
     </row>
     <row r="184" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A184" s="10"/>
@@ -4662,9 +4643,9 @@
       </c>
       <c r="C184" s="10"/>
       <c r="D184" s="27" t="s">
-        <v>314</v>
-      </c>
-      <c r="E184" s="61"/>
+        <v>311</v>
+      </c>
+      <c r="E184" s="63"/>
     </row>
     <row r="185" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A185" s="10"/>
@@ -4677,7 +4658,7 @@
       <c r="D185" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="E185" s="61"/>
+      <c r="E185" s="63"/>
     </row>
     <row r="186" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A186" s="10"/>
@@ -4690,7 +4671,7 @@
       <c r="D186" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="E186" s="61"/>
+      <c r="E186" s="63"/>
     </row>
     <row r="187" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A187" s="10"/>
@@ -4701,7 +4682,7 @@
       <c r="D187" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="E187" s="61"/>
+      <c r="E187" s="63"/>
     </row>
     <row r="188" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A188" s="28"/>
@@ -4712,7 +4693,7 @@
       <c r="D188" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="E188" s="62"/>
+      <c r="E188" s="64"/>
     </row>
     <row r="189" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A189" s="10"/>
@@ -4727,7 +4708,7 @@
       <c r="B190" s="57"/>
       <c r="C190" s="10"/>
       <c r="D190" s="11"/>
-      <c r="E190" s="61" t="s">
+      <c r="E190" s="63" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4736,7 +4717,7 @@
       <c r="B191" s="57"/>
       <c r="C191" s="10"/>
       <c r="D191" s="13"/>
-      <c r="E191" s="61"/>
+      <c r="E191" s="63"/>
     </row>
     <row r="192" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A192" s="14" t="s">
@@ -4745,21 +4726,21 @@
       <c r="B192" s="57"/>
       <c r="C192" s="10"/>
       <c r="D192" s="13"/>
-      <c r="E192" s="61"/>
+      <c r="E192" s="63"/>
     </row>
     <row r="193" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A193" s="15"/>
       <c r="B193" s="57"/>
       <c r="C193" s="10"/>
       <c r="D193" s="13"/>
-      <c r="E193" s="61"/>
+      <c r="E193" s="63"/>
     </row>
     <row r="194" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A194" s="15"/>
       <c r="B194" s="57"/>
       <c r="C194" s="10"/>
       <c r="D194" s="13"/>
-      <c r="E194" s="61"/>
+      <c r="E194" s="63"/>
     </row>
     <row r="195" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A195" s="23" t="s">
@@ -4768,13 +4749,13 @@
       <c r="B195" s="57" t="s">
         <v>134</v>
       </c>
-      <c r="C195" s="74" t="s">
+      <c r="C195" s="59" t="s">
         <v>135</v>
       </c>
       <c r="D195" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="E195" s="61"/>
+      <c r="E195" s="63"/>
     </row>
     <row r="196" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A196" s="23" t="s">
@@ -4783,98 +4764,98 @@
       <c r="B196" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="C196" s="74" t="s">
+      <c r="C196" s="59" t="s">
         <v>139</v>
       </c>
       <c r="D196" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="E196" s="61"/>
+      <c r="E196" s="63"/>
     </row>
     <row r="197" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A197" s="15"/>
       <c r="B197" s="57"/>
       <c r="C197" s="10"/>
       <c r="D197" s="13"/>
-      <c r="E197" s="61"/>
+      <c r="E197" s="63"/>
     </row>
     <row r="198" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A198" s="15"/>
       <c r="B198" s="57"/>
       <c r="C198" s="10"/>
       <c r="D198" s="13"/>
-      <c r="E198" s="61"/>
+      <c r="E198" s="63"/>
     </row>
     <row r="199" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A199" s="15" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B199" s="57" t="s">
-        <v>308</v>
-      </c>
-      <c r="C199" s="78" t="s">
-        <v>309</v>
+        <v>305</v>
+      </c>
+      <c r="C199" s="61" t="s">
+        <v>306</v>
       </c>
       <c r="D199" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="E199" s="61"/>
+        <v>307</v>
+      </c>
+      <c r="E199" s="63"/>
     </row>
     <row r="200" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A200" s="15"/>
       <c r="B200" s="57"/>
       <c r="C200" s="10"/>
       <c r="D200" s="13"/>
-      <c r="E200" s="61"/>
+      <c r="E200" s="63"/>
     </row>
     <row r="201" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A201" s="10"/>
       <c r="B201" s="58"/>
       <c r="C201" s="18"/>
       <c r="D201" s="13"/>
-      <c r="E201" s="61"/>
+      <c r="E201" s="63"/>
     </row>
     <row r="202" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A202" s="23"/>
       <c r="B202" s="57"/>
       <c r="C202" s="18"/>
       <c r="D202" s="13"/>
-      <c r="E202" s="61"/>
+      <c r="E202" s="63"/>
     </row>
     <row r="203" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A203" s="23"/>
       <c r="B203" s="57"/>
       <c r="C203" s="18"/>
       <c r="D203" s="13"/>
-      <c r="E203" s="61"/>
+      <c r="E203" s="63"/>
     </row>
     <row r="204" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A204" s="23"/>
       <c r="B204" s="57"/>
       <c r="C204" s="18"/>
       <c r="D204" s="13"/>
-      <c r="E204" s="61"/>
+      <c r="E204" s="63"/>
     </row>
     <row r="205" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A205" s="23"/>
       <c r="B205" s="57"/>
       <c r="C205" s="18"/>
       <c r="D205" s="13"/>
-      <c r="E205" s="61"/>
+      <c r="E205" s="63"/>
     </row>
     <row r="206" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A206" s="21"/>
       <c r="B206" s="58"/>
       <c r="C206" s="20"/>
       <c r="D206" s="13"/>
-      <c r="E206" s="61"/>
+      <c r="E206" s="63"/>
     </row>
     <row r="207" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A207" s="10"/>
       <c r="B207" s="57"/>
       <c r="C207" s="10"/>
       <c r="D207" s="13"/>
-      <c r="E207" s="61"/>
+      <c r="E207" s="63"/>
     </row>
     <row r="208" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A208" s="10"/>
@@ -4885,7 +4866,7 @@
       <c r="D208" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="E208" s="61"/>
+      <c r="E208" s="63"/>
     </row>
     <row r="209" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A209" s="10"/>
@@ -4898,7 +4879,7 @@
       <c r="D209" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="E209" s="61"/>
+      <c r="E209" s="63"/>
     </row>
     <row r="210" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A210" s="10"/>
@@ -4911,7 +4892,7 @@
       <c r="D210" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="E210" s="61"/>
+      <c r="E210" s="63"/>
     </row>
     <row r="211" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A211" s="10"/>
@@ -4922,7 +4903,7 @@
       <c r="D211" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="E211" s="61"/>
+      <c r="E211" s="63"/>
     </row>
     <row r="212" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A212" s="28"/>
@@ -4933,7 +4914,7 @@
       <c r="D212" s="30" t="s">
         <v>145</v>
       </c>
-      <c r="E212" s="62"/>
+      <c r="E212" s="64"/>
     </row>
     <row r="213" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A213" s="10"/>
@@ -4948,8 +4929,8 @@
       <c r="B214" s="10"/>
       <c r="C214" s="10"/>
       <c r="D214" s="11"/>
-      <c r="E214" s="61" t="s">
-        <v>316</v>
+      <c r="E214" s="63" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="215" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
@@ -4957,7 +4938,7 @@
       <c r="B215" s="10"/>
       <c r="C215" s="10"/>
       <c r="D215" s="13"/>
-      <c r="E215" s="61"/>
+      <c r="E215" s="63"/>
     </row>
     <row r="216" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A216" s="14" t="s">
@@ -4966,30 +4947,30 @@
       <c r="B216" s="10"/>
       <c r="C216" s="10"/>
       <c r="D216" s="13"/>
-      <c r="E216" s="61"/>
+      <c r="E216" s="63"/>
     </row>
     <row r="217" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A217" s="41"/>
       <c r="B217" s="10"/>
       <c r="C217" s="10"/>
       <c r="D217" s="13"/>
-      <c r="E217" s="61"/>
+      <c r="E217" s="63"/>
     </row>
     <row r="218" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A218" s="14" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B218" s="36"/>
       <c r="C218" s="42"/>
       <c r="D218" s="13"/>
-      <c r="E218" s="61"/>
+      <c r="E218" s="63"/>
     </row>
     <row r="219" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A219" s="41"/>
       <c r="B219" s="36"/>
       <c r="C219" s="42"/>
       <c r="D219" s="13"/>
-      <c r="E219" s="61"/>
+      <c r="E219" s="63"/>
     </row>
     <row r="220" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A220" s="41" t="s">
@@ -5000,163 +4981,167 @@
       </c>
       <c r="C220" s="42"/>
       <c r="D220" s="13"/>
-      <c r="E220" s="61"/>
+      <c r="E220" s="63"/>
     </row>
     <row r="221" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A221" s="41" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B221" s="36" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C221" s="42"/>
       <c r="D221" s="13"/>
-      <c r="E221" s="61"/>
+      <c r="E221" s="63"/>
     </row>
     <row r="222" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A222" s="41" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B222" s="36" t="s">
-        <v>321</v>
-      </c>
-      <c r="C222" s="77" t="s">
-        <v>322</v>
+        <v>317</v>
+      </c>
+      <c r="C222" s="59" t="s">
+        <v>318</v>
       </c>
       <c r="D222" s="13" t="s">
-        <v>323</v>
-      </c>
-      <c r="E222" s="61"/>
+        <v>319</v>
+      </c>
+      <c r="E222" s="63"/>
     </row>
     <row r="223" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A223" s="41"/>
-      <c r="B223" s="36"/>
+      <c r="B223" s="36" t="s">
+        <v>332</v>
+      </c>
       <c r="C223" s="42"/>
-      <c r="D223" s="13"/>
-      <c r="E223" s="61"/>
+      <c r="D223" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="E223" s="63"/>
     </row>
     <row r="224" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A224" s="41"/>
       <c r="B224" s="36"/>
       <c r="C224" s="42"/>
       <c r="D224" s="13"/>
-      <c r="E224" s="61"/>
+      <c r="E224" s="63"/>
     </row>
     <row r="225" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A225" s="41"/>
       <c r="B225" s="36"/>
       <c r="C225" s="42"/>
       <c r="D225" s="13"/>
-      <c r="E225" s="61"/>
+      <c r="E225" s="63"/>
     </row>
     <row r="226" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A226" s="41"/>
       <c r="B226" s="36"/>
       <c r="C226" s="42"/>
       <c r="D226" s="13"/>
-      <c r="E226" s="61"/>
+      <c r="E226" s="63"/>
     </row>
     <row r="227" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A227" s="41"/>
       <c r="B227" s="36"/>
       <c r="C227" s="42"/>
       <c r="D227" s="13"/>
-      <c r="E227" s="61"/>
+      <c r="E227" s="63"/>
     </row>
     <row r="228" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A228" s="41"/>
       <c r="B228" s="36"/>
       <c r="C228" s="42"/>
       <c r="D228" s="13"/>
-      <c r="E228" s="61"/>
+      <c r="E228" s="63"/>
     </row>
     <row r="229" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A229" s="41"/>
       <c r="B229" s="36"/>
       <c r="C229" s="42"/>
       <c r="D229" s="13"/>
-      <c r="E229" s="61"/>
+      <c r="E229" s="63"/>
     </row>
     <row r="230" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A230" s="41"/>
       <c r="B230" s="36"/>
       <c r="C230" s="42"/>
       <c r="D230" s="13"/>
-      <c r="E230" s="61"/>
+      <c r="E230" s="63"/>
     </row>
     <row r="231" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A231" s="41"/>
       <c r="B231" s="36"/>
       <c r="C231" s="42"/>
       <c r="D231" s="13"/>
-      <c r="E231" s="61"/>
+      <c r="E231" s="63"/>
     </row>
     <row r="232" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A232" s="41"/>
       <c r="B232" s="36"/>
       <c r="C232" s="42"/>
       <c r="D232" s="13"/>
-      <c r="E232" s="61"/>
+      <c r="E232" s="63"/>
     </row>
     <row r="233" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A233" s="41"/>
       <c r="B233" s="36"/>
       <c r="C233" s="42"/>
       <c r="D233" s="13"/>
-      <c r="E233" s="61"/>
+      <c r="E233" s="63"/>
     </row>
     <row r="234" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A234" s="21"/>
       <c r="B234" s="17"/>
       <c r="C234" s="43"/>
       <c r="D234" s="27"/>
-      <c r="E234" s="61"/>
+      <c r="E234" s="63"/>
     </row>
     <row r="235" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A235" s="21"/>
       <c r="B235" s="17"/>
       <c r="C235" s="43"/>
       <c r="D235" s="27"/>
-      <c r="E235" s="61"/>
+      <c r="E235" s="63"/>
     </row>
     <row r="236" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A236" s="10"/>
       <c r="B236" s="44"/>
       <c r="C236" s="42"/>
       <c r="D236" s="13"/>
-      <c r="E236" s="61"/>
+      <c r="E236" s="63"/>
     </row>
     <row r="237" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A237" s="10"/>
       <c r="B237" s="44"/>
       <c r="C237" s="42"/>
       <c r="D237" s="13"/>
-      <c r="E237" s="61"/>
+      <c r="E237" s="63"/>
     </row>
     <row r="238" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A238" s="10"/>
       <c r="B238" s="44"/>
       <c r="C238" s="42"/>
       <c r="D238" s="13"/>
-      <c r="E238" s="61"/>
+      <c r="E238" s="63"/>
     </row>
     <row r="239" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A239" s="21" t="s">
         <v>48</v>
       </c>
       <c r="B239" s="17" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C239" s="20"/>
       <c r="D239" s="13"/>
-      <c r="E239" s="61"/>
+      <c r="E239" s="63"/>
     </row>
     <row r="240" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A240" s="10"/>
       <c r="B240" s="10"/>
       <c r="C240" s="10"/>
       <c r="D240" s="13"/>
-      <c r="E240" s="61"/>
+      <c r="E240" s="63"/>
     </row>
     <row r="241" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A241" s="10"/>
@@ -5167,7 +5152,7 @@
       <c r="D241" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="E241" s="61"/>
+      <c r="E241" s="63"/>
     </row>
     <row r="242" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A242" s="10"/>
@@ -5180,7 +5165,7 @@
       <c r="D242" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="E242" s="61"/>
+      <c r="E242" s="63"/>
     </row>
     <row r="243" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A243" s="10"/>
@@ -5193,7 +5178,7 @@
       <c r="D243" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="E243" s="61"/>
+      <c r="E243" s="63"/>
     </row>
     <row r="244" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A244" s="10"/>
@@ -5206,7 +5191,7 @@
       <c r="D244" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="E244" s="61"/>
+      <c r="E244" s="63"/>
     </row>
     <row r="245" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A245" s="28"/>
@@ -5232,7 +5217,7 @@
       <c r="B247" s="10"/>
       <c r="C247" s="10"/>
       <c r="D247" s="11"/>
-      <c r="E247" s="60" t="s">
+      <c r="E247" s="62" t="s">
         <v>156</v>
       </c>
     </row>
@@ -5241,7 +5226,7 @@
       <c r="B248" s="10"/>
       <c r="C248" s="10"/>
       <c r="D248" s="46"/>
-      <c r="E248" s="61"/>
+      <c r="E248" s="63"/>
     </row>
     <row r="249" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A249" s="14" t="s">
@@ -5250,7 +5235,7 @@
       <c r="B249" s="10"/>
       <c r="C249" s="10"/>
       <c r="D249" s="13"/>
-      <c r="E249" s="61"/>
+      <c r="E249" s="63"/>
     </row>
     <row r="250" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A250" s="14" t="s">
@@ -5259,13 +5244,13 @@
       <c r="B250" s="36" t="s">
         <v>159</v>
       </c>
-      <c r="C250" s="77" t="s">
+      <c r="C250" s="59" t="s">
         <v>160</v>
       </c>
       <c r="D250" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="E250" s="61"/>
+      <c r="E250" s="63"/>
     </row>
     <row r="251" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A251" s="41" t="s">
@@ -5276,7 +5261,7 @@
       </c>
       <c r="C251" s="42"/>
       <c r="D251" s="13"/>
-      <c r="E251" s="61"/>
+      <c r="E251" s="63"/>
     </row>
     <row r="252" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A252" s="41" t="s">
@@ -5287,14 +5272,14 @@
       </c>
       <c r="C252" s="42"/>
       <c r="D252" s="13"/>
-      <c r="E252" s="61"/>
+      <c r="E252" s="63"/>
     </row>
     <row r="253" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A253" s="41"/>
       <c r="B253" s="36"/>
       <c r="C253" s="42"/>
       <c r="D253" s="13"/>
-      <c r="E253" s="61"/>
+      <c r="E253" s="63"/>
     </row>
     <row r="254" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A254" s="14" t="s">
@@ -5303,70 +5288,70 @@
       <c r="B254" s="36"/>
       <c r="C254" s="42"/>
       <c r="D254" s="13"/>
-      <c r="E254" s="61"/>
+      <c r="E254" s="63"/>
     </row>
     <row r="255" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A255" s="41"/>
       <c r="B255" s="36"/>
       <c r="C255" s="42"/>
       <c r="D255" s="13"/>
-      <c r="E255" s="61"/>
+      <c r="E255" s="63"/>
     </row>
     <row r="256" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A256" s="41"/>
       <c r="B256" s="36"/>
       <c r="C256" s="42"/>
       <c r="D256" s="13"/>
-      <c r="E256" s="61"/>
+      <c r="E256" s="63"/>
     </row>
     <row r="257" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A257" s="41"/>
       <c r="B257" s="36"/>
       <c r="C257" s="42"/>
       <c r="D257" s="13"/>
-      <c r="E257" s="61"/>
+      <c r="E257" s="63"/>
     </row>
     <row r="258" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A258" s="41"/>
       <c r="B258" s="36"/>
       <c r="C258" s="42"/>
       <c r="D258" s="13"/>
-      <c r="E258" s="61"/>
+      <c r="E258" s="63"/>
     </row>
     <row r="259" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A259" s="21"/>
       <c r="B259" s="17"/>
       <c r="C259" s="43"/>
       <c r="D259" s="27"/>
-      <c r="E259" s="61"/>
+      <c r="E259" s="63"/>
     </row>
     <row r="260" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A260" s="21"/>
       <c r="B260" s="17"/>
       <c r="C260" s="43"/>
       <c r="D260" s="27"/>
-      <c r="E260" s="61"/>
+      <c r="E260" s="63"/>
     </row>
     <row r="261" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A261" s="10"/>
       <c r="B261" s="44"/>
       <c r="C261" s="42"/>
       <c r="D261" s="13"/>
-      <c r="E261" s="61"/>
+      <c r="E261" s="63"/>
     </row>
     <row r="262" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A262" s="10"/>
       <c r="B262" s="44"/>
       <c r="C262" s="42"/>
       <c r="D262" s="13"/>
-      <c r="E262" s="61"/>
+      <c r="E262" s="63"/>
     </row>
     <row r="263" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A263" s="10"/>
       <c r="B263" s="44"/>
       <c r="C263" s="42"/>
       <c r="D263" s="13"/>
-      <c r="E263" s="61"/>
+      <c r="E263" s="63"/>
     </row>
     <row r="264" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A264" s="21" t="s">
@@ -5377,14 +5362,14 @@
       </c>
       <c r="C264" s="20"/>
       <c r="D264" s="13"/>
-      <c r="E264" s="61"/>
+      <c r="E264" s="63"/>
     </row>
     <row r="265" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A265" s="10"/>
       <c r="B265" s="10"/>
       <c r="C265" s="10"/>
       <c r="D265" s="13"/>
-      <c r="E265" s="61"/>
+      <c r="E265" s="63"/>
     </row>
     <row r="266" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A266" s="10"/>
@@ -5395,7 +5380,7 @@
       <c r="D266" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="E266" s="61"/>
+      <c r="E266" s="63"/>
     </row>
     <row r="267" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A267" s="10"/>
@@ -5408,7 +5393,7 @@
       <c r="D267" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="E267" s="61"/>
+      <c r="E267" s="63"/>
     </row>
     <row r="268" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A268" s="10"/>
@@ -5421,7 +5406,7 @@
       <c r="D268" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="E268" s="61"/>
+      <c r="E268" s="63"/>
     </row>
     <row r="269" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A269" s="10"/>
@@ -5432,7 +5417,7 @@
       <c r="D269" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="E269" s="61"/>
+      <c r="E269" s="63"/>
     </row>
     <row r="270" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A270" s="28"/>
@@ -5458,7 +5443,7 @@
       <c r="B272" s="10"/>
       <c r="C272" s="10"/>
       <c r="D272" s="11"/>
-      <c r="E272" s="60" t="s">
+      <c r="E272" s="62" t="s">
         <v>172</v>
       </c>
     </row>
@@ -5467,7 +5452,7 @@
       <c r="B273" s="10"/>
       <c r="C273" s="10"/>
       <c r="D273" s="46"/>
-      <c r="E273" s="61"/>
+      <c r="E273" s="63"/>
     </row>
     <row r="274" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A274" s="14" t="s">
@@ -5476,7 +5461,7 @@
       <c r="B274" s="10"/>
       <c r="C274" s="10"/>
       <c r="D274" s="13"/>
-      <c r="E274" s="61"/>
+      <c r="E274" s="63"/>
     </row>
     <row r="275" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A275" s="14" t="s">
@@ -5485,13 +5470,13 @@
       <c r="B275" s="36" t="s">
         <v>159</v>
       </c>
-      <c r="C275" s="77" t="s">
+      <c r="C275" s="59" t="s">
         <v>160</v>
       </c>
       <c r="D275" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="E275" s="61"/>
+      <c r="E275" s="63"/>
     </row>
     <row r="276" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A276" s="41" t="s">
@@ -5502,7 +5487,7 @@
       </c>
       <c r="C276" s="42"/>
       <c r="D276" s="13"/>
-      <c r="E276" s="61"/>
+      <c r="E276" s="63"/>
     </row>
     <row r="277" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A277" s="41" t="s">
@@ -5513,14 +5498,14 @@
       </c>
       <c r="C277" s="42"/>
       <c r="D277" s="13"/>
-      <c r="E277" s="61"/>
+      <c r="E277" s="63"/>
     </row>
     <row r="278" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A278" s="41"/>
       <c r="B278" s="36"/>
       <c r="C278" s="42"/>
       <c r="D278" s="13"/>
-      <c r="E278" s="61"/>
+      <c r="E278" s="63"/>
     </row>
     <row r="279" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A279" s="14" t="s">
@@ -5529,70 +5514,70 @@
       <c r="B279" s="36"/>
       <c r="C279" s="42"/>
       <c r="D279" s="13"/>
-      <c r="E279" s="61"/>
+      <c r="E279" s="63"/>
     </row>
     <row r="280" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A280" s="41"/>
       <c r="B280" s="36"/>
       <c r="C280" s="42"/>
       <c r="D280" s="13"/>
-      <c r="E280" s="61"/>
+      <c r="E280" s="63"/>
     </row>
     <row r="281" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A281" s="41"/>
       <c r="B281" s="36"/>
       <c r="C281" s="42"/>
       <c r="D281" s="13"/>
-      <c r="E281" s="61"/>
+      <c r="E281" s="63"/>
     </row>
     <row r="282" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A282" s="41"/>
       <c r="B282" s="36"/>
       <c r="C282" s="42"/>
       <c r="D282" s="13"/>
-      <c r="E282" s="61"/>
+      <c r="E282" s="63"/>
     </row>
     <row r="283" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A283" s="41"/>
       <c r="B283" s="36"/>
       <c r="C283" s="42"/>
       <c r="D283" s="13"/>
-      <c r="E283" s="61"/>
+      <c r="E283" s="63"/>
     </row>
     <row r="284" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A284" s="21"/>
       <c r="B284" s="17"/>
       <c r="C284" s="43"/>
       <c r="D284" s="27"/>
-      <c r="E284" s="61"/>
+      <c r="E284" s="63"/>
     </row>
     <row r="285" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A285" s="21"/>
       <c r="B285" s="17"/>
       <c r="C285" s="43"/>
       <c r="D285" s="27"/>
-      <c r="E285" s="61"/>
+      <c r="E285" s="63"/>
     </row>
     <row r="286" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A286" s="10"/>
       <c r="B286" s="44"/>
       <c r="C286" s="42"/>
       <c r="D286" s="13"/>
-      <c r="E286" s="61"/>
+      <c r="E286" s="63"/>
     </row>
     <row r="287" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A287" s="10"/>
       <c r="B287" s="44"/>
       <c r="C287" s="42"/>
       <c r="D287" s="13"/>
-      <c r="E287" s="61"/>
+      <c r="E287" s="63"/>
     </row>
     <row r="288" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A288" s="10"/>
       <c r="B288" s="44"/>
       <c r="C288" s="42"/>
       <c r="D288" s="13"/>
-      <c r="E288" s="61"/>
+      <c r="E288" s="63"/>
     </row>
     <row r="289" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A289" s="21" t="s">
@@ -5603,14 +5588,14 @@
       </c>
       <c r="C289" s="20"/>
       <c r="D289" s="13"/>
-      <c r="E289" s="61"/>
+      <c r="E289" s="63"/>
     </row>
     <row r="290" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A290" s="10"/>
       <c r="B290" s="10"/>
       <c r="C290" s="10"/>
       <c r="D290" s="13"/>
-      <c r="E290" s="61"/>
+      <c r="E290" s="63"/>
     </row>
     <row r="291" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A291" s="10"/>
@@ -5621,7 +5606,7 @@
       <c r="D291" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="E291" s="61"/>
+      <c r="E291" s="63"/>
     </row>
     <row r="292" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A292" s="10"/>
@@ -5634,7 +5619,7 @@
       <c r="D292" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="E292" s="61"/>
+      <c r="E292" s="63"/>
     </row>
     <row r="293" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A293" s="10"/>
@@ -5647,7 +5632,7 @@
       <c r="D293" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="E293" s="61"/>
+      <c r="E293" s="63"/>
     </row>
     <row r="294" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A294" s="10"/>
@@ -5658,7 +5643,7 @@
       <c r="D294" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="E294" s="61"/>
+      <c r="E294" s="63"/>
     </row>
     <row r="295" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A295" s="28"/>
@@ -5684,7 +5669,7 @@
       <c r="B297" s="10"/>
       <c r="C297" s="10"/>
       <c r="D297" s="11"/>
-      <c r="E297" s="60" t="s">
+      <c r="E297" s="62" t="s">
         <v>175</v>
       </c>
     </row>
@@ -5693,7 +5678,7 @@
       <c r="B298" s="10"/>
       <c r="C298" s="10"/>
       <c r="D298" s="46"/>
-      <c r="E298" s="61"/>
+      <c r="E298" s="63"/>
     </row>
     <row r="299" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A299" s="14" t="s">
@@ -5702,27 +5687,27 @@
       <c r="B299" s="10"/>
       <c r="C299" s="10"/>
       <c r="D299" s="13"/>
-      <c r="E299" s="61"/>
+      <c r="E299" s="63"/>
     </row>
     <row r="300" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A300" s="14"/>
       <c r="C300" s="36"/>
       <c r="D300" s="13"/>
-      <c r="E300" s="61"/>
+      <c r="E300" s="63"/>
     </row>
     <row r="301" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A301" s="41"/>
       <c r="B301" s="36"/>
       <c r="C301" s="42"/>
       <c r="D301" s="13"/>
-      <c r="E301" s="61"/>
+      <c r="E301" s="63"/>
     </row>
     <row r="302" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A302" s="41"/>
       <c r="B302" s="36"/>
       <c r="C302" s="42"/>
       <c r="D302" s="13"/>
-      <c r="E302" s="61"/>
+      <c r="E302" s="63"/>
     </row>
     <row r="303" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A303" s="41"/>
@@ -5735,7 +5720,7 @@
       <c r="D303" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="E303" s="61"/>
+      <c r="E303" s="63"/>
     </row>
     <row r="304" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A304" s="14" t="s">
@@ -5744,84 +5729,84 @@
       <c r="B304" s="36"/>
       <c r="C304" s="42"/>
       <c r="D304" s="13"/>
-      <c r="E304" s="61"/>
+      <c r="E304" s="63"/>
     </row>
     <row r="305" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A305" s="41"/>
       <c r="B305" s="36"/>
       <c r="C305" s="42"/>
       <c r="D305" s="13"/>
-      <c r="E305" s="61"/>
+      <c r="E305" s="63"/>
     </row>
     <row r="306" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A306" s="41"/>
       <c r="B306" s="36"/>
       <c r="C306" s="42"/>
       <c r="D306" s="13"/>
-      <c r="E306" s="61"/>
+      <c r="E306" s="63"/>
     </row>
     <row r="307" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A307" s="41"/>
       <c r="B307" s="36"/>
       <c r="C307" s="42"/>
       <c r="D307" s="13"/>
-      <c r="E307" s="61"/>
+      <c r="E307" s="63"/>
     </row>
     <row r="308" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A308" s="41"/>
       <c r="B308" s="36"/>
       <c r="C308" s="42"/>
       <c r="D308" s="13"/>
-      <c r="E308" s="61"/>
+      <c r="E308" s="63"/>
     </row>
     <row r="309" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A309" s="21"/>
       <c r="B309" s="17"/>
       <c r="C309" s="43"/>
       <c r="D309" s="27"/>
-      <c r="E309" s="61"/>
+      <c r="E309" s="63"/>
     </row>
     <row r="310" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A310" s="21"/>
       <c r="B310" s="17"/>
       <c r="C310" s="43"/>
       <c r="D310" s="27"/>
-      <c r="E310" s="61"/>
+      <c r="E310" s="63"/>
     </row>
     <row r="311" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A311" s="10"/>
       <c r="B311" s="44"/>
       <c r="C311" s="42"/>
       <c r="D311" s="13"/>
-      <c r="E311" s="61"/>
+      <c r="E311" s="63"/>
     </row>
     <row r="312" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A312" s="10"/>
       <c r="B312" s="44"/>
       <c r="C312" s="42"/>
       <c r="D312" s="13"/>
-      <c r="E312" s="61"/>
+      <c r="E312" s="63"/>
     </row>
     <row r="313" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A313" s="10"/>
       <c r="B313" s="44"/>
       <c r="C313" s="42"/>
       <c r="D313" s="13"/>
-      <c r="E313" s="61"/>
+      <c r="E313" s="63"/>
     </row>
     <row r="314" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A314" s="21"/>
       <c r="B314" s="17"/>
       <c r="C314" s="20"/>
       <c r="D314" s="13"/>
-      <c r="E314" s="61"/>
+      <c r="E314" s="63"/>
     </row>
     <row r="315" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A315" s="10"/>
       <c r="B315" s="10"/>
       <c r="C315" s="10"/>
       <c r="D315" s="13"/>
-      <c r="E315" s="61"/>
+      <c r="E315" s="63"/>
     </row>
     <row r="316" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A316" s="10"/>
@@ -5832,7 +5817,7 @@
       <c r="D316" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="E316" s="61"/>
+      <c r="E316" s="63"/>
     </row>
     <row r="317" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A317" s="10"/>
@@ -5845,7 +5830,7 @@
       <c r="D317" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="E317" s="61"/>
+      <c r="E317" s="63"/>
     </row>
     <row r="318" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A318" s="10"/>
@@ -5858,7 +5843,7 @@
       <c r="D318" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="E318" s="61"/>
+      <c r="E318" s="63"/>
     </row>
     <row r="319" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A319" s="10"/>
@@ -5869,7 +5854,7 @@
       <c r="D319" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="E319" s="61"/>
+      <c r="E319" s="63"/>
     </row>
     <row r="320" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A320" s="28"/>
@@ -5895,7 +5880,7 @@
       <c r="B322" s="10"/>
       <c r="C322" s="10"/>
       <c r="D322" s="11"/>
-      <c r="E322" s="60" t="s">
+      <c r="E322" s="62" t="s">
         <v>179</v>
       </c>
     </row>
@@ -5904,7 +5889,7 @@
       <c r="B323" s="10"/>
       <c r="C323" s="10"/>
       <c r="D323" s="46"/>
-      <c r="E323" s="61"/>
+      <c r="E323" s="63"/>
     </row>
     <row r="324" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A324" s="14" t="s">
@@ -5913,13 +5898,13 @@
       <c r="B324" s="10"/>
       <c r="C324" s="10"/>
       <c r="D324" s="13"/>
-      <c r="E324" s="61"/>
+      <c r="E324" s="63"/>
     </row>
     <row r="325" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A325" s="14"/>
       <c r="C325" s="36"/>
       <c r="D325" s="13"/>
-      <c r="E325" s="61"/>
+      <c r="E325" s="63"/>
     </row>
     <row r="326" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A326" s="14" t="s">
@@ -5932,21 +5917,21 @@
       <c r="D326" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="E326" s="61"/>
+      <c r="E326" s="63"/>
     </row>
     <row r="327" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A327" s="41"/>
       <c r="B327" s="36"/>
       <c r="C327" s="42"/>
       <c r="D327" s="13"/>
-      <c r="E327" s="61"/>
+      <c r="E327" s="63"/>
     </row>
     <row r="328" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A328" s="41"/>
       <c r="B328" s="36"/>
       <c r="C328" s="34"/>
       <c r="D328" s="13"/>
-      <c r="E328" s="61"/>
+      <c r="E328" s="63"/>
     </row>
     <row r="329" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A329" s="14" t="s">
@@ -5955,84 +5940,84 @@
       <c r="B329" s="36"/>
       <c r="C329" s="42"/>
       <c r="D329" s="13"/>
-      <c r="E329" s="61"/>
+      <c r="E329" s="63"/>
     </row>
     <row r="330" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A330" s="41"/>
       <c r="B330" s="36"/>
       <c r="C330" s="42"/>
       <c r="D330" s="13"/>
-      <c r="E330" s="61"/>
+      <c r="E330" s="63"/>
     </row>
     <row r="331" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A331" s="41"/>
       <c r="B331" s="36"/>
       <c r="C331" s="42"/>
       <c r="D331" s="13"/>
-      <c r="E331" s="61"/>
+      <c r="E331" s="63"/>
     </row>
     <row r="332" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A332" s="41"/>
       <c r="B332" s="36"/>
       <c r="C332" s="42"/>
       <c r="D332" s="13"/>
-      <c r="E332" s="61"/>
+      <c r="E332" s="63"/>
     </row>
     <row r="333" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A333" s="41"/>
       <c r="B333" s="36"/>
       <c r="C333" s="42"/>
       <c r="D333" s="13"/>
-      <c r="E333" s="61"/>
+      <c r="E333" s="63"/>
     </row>
     <row r="334" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A334" s="21"/>
       <c r="B334" s="17"/>
       <c r="C334" s="43"/>
       <c r="D334" s="27"/>
-      <c r="E334" s="61"/>
+      <c r="E334" s="63"/>
     </row>
     <row r="335" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A335" s="21"/>
       <c r="B335" s="17"/>
       <c r="C335" s="43"/>
       <c r="D335" s="27"/>
-      <c r="E335" s="61"/>
+      <c r="E335" s="63"/>
     </row>
     <row r="336" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A336" s="10"/>
       <c r="B336" s="44"/>
       <c r="C336" s="42"/>
       <c r="D336" s="13"/>
-      <c r="E336" s="61"/>
+      <c r="E336" s="63"/>
     </row>
     <row r="337" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A337" s="10"/>
       <c r="B337" s="44"/>
       <c r="C337" s="42"/>
       <c r="D337" s="13"/>
-      <c r="E337" s="61"/>
+      <c r="E337" s="63"/>
     </row>
     <row r="338" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A338" s="10"/>
       <c r="B338" s="44"/>
       <c r="C338" s="42"/>
       <c r="D338" s="13"/>
-      <c r="E338" s="61"/>
+      <c r="E338" s="63"/>
     </row>
     <row r="339" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A339" s="21"/>
       <c r="B339" s="17"/>
       <c r="C339" s="20"/>
       <c r="D339" s="13"/>
-      <c r="E339" s="61"/>
+      <c r="E339" s="63"/>
     </row>
     <row r="340" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A340" s="10"/>
       <c r="B340" s="10"/>
       <c r="C340" s="10"/>
       <c r="D340" s="13"/>
-      <c r="E340" s="61"/>
+      <c r="E340" s="63"/>
     </row>
     <row r="341" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A341" s="10"/>
@@ -6043,7 +6028,7 @@
       <c r="D341" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="E341" s="61"/>
+      <c r="E341" s="63"/>
     </row>
     <row r="342" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A342" s="10"/>
@@ -6056,7 +6041,7 @@
       <c r="D342" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="E342" s="61"/>
+      <c r="E342" s="63"/>
     </row>
     <row r="343" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A343" s="10"/>
@@ -6069,7 +6054,7 @@
       <c r="D343" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="E343" s="61"/>
+      <c r="E343" s="63"/>
     </row>
     <row r="344" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A344" s="10"/>
@@ -6080,7 +6065,7 @@
       <c r="D344" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="E344" s="61"/>
+      <c r="E344" s="63"/>
     </row>
     <row r="345" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A345" s="28"/>
@@ -6106,7 +6091,7 @@
       <c r="B347" s="19"/>
       <c r="C347" s="18"/>
       <c r="D347" s="13"/>
-      <c r="E347" s="61" t="s">
+      <c r="E347" s="63" t="s">
         <v>184</v>
       </c>
     </row>
@@ -6115,7 +6100,7 @@
       <c r="B348" s="19"/>
       <c r="C348" s="18"/>
       <c r="D348" s="13"/>
-      <c r="E348" s="61"/>
+      <c r="E348" s="63"/>
     </row>
     <row r="349" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A349" s="10" t="s">
@@ -6124,14 +6109,14 @@
       <c r="B349" s="17"/>
       <c r="C349" s="18"/>
       <c r="D349" s="13"/>
-      <c r="E349" s="61"/>
+      <c r="E349" s="63"/>
     </row>
     <row r="350" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A350" s="10"/>
       <c r="B350" s="17"/>
       <c r="C350" s="18"/>
       <c r="D350" s="13"/>
-      <c r="E350" s="61"/>
+      <c r="E350" s="63"/>
     </row>
     <row r="351" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A351" s="10" t="s">
@@ -6140,13 +6125,13 @@
       <c r="B351" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="C351" s="73" t="s">
+      <c r="C351" s="59" t="s">
         <v>188</v>
       </c>
       <c r="D351" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="E351" s="61"/>
+      <c r="E351" s="63"/>
     </row>
     <row r="352" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A352" s="10" t="s">
@@ -6155,13 +6140,13 @@
       <c r="B352" s="17" t="s">
         <v>191</v>
       </c>
-      <c r="C352" s="73" t="s">
+      <c r="C352" s="59" t="s">
         <v>192</v>
       </c>
       <c r="D352" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="E352" s="61"/>
+      <c r="E352" s="63"/>
     </row>
     <row r="353" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A353" s="10" t="s">
@@ -6170,13 +6155,13 @@
       <c r="B353" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="C353" s="74" t="s">
+      <c r="C353" s="59" t="s">
         <v>196</v>
       </c>
       <c r="D353" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="E353" s="61"/>
+      <c r="E353" s="63"/>
     </row>
     <row r="354" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A354" s="10" t="s">
@@ -6185,13 +6170,13 @@
       <c r="B354" s="17" t="s">
         <v>199</v>
       </c>
-      <c r="C354" s="74" t="s">
+      <c r="C354" s="59" t="s">
         <v>200</v>
       </c>
       <c r="D354" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="E354" s="61"/>
+      <c r="E354" s="63"/>
     </row>
     <row r="355" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A355" s="10" t="s">
@@ -6200,27 +6185,27 @@
       <c r="B355" s="17" t="s">
         <v>203</v>
       </c>
-      <c r="C355" s="74" t="s">
+      <c r="C355" s="59" t="s">
         <v>204</v>
       </c>
       <c r="D355" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="E355" s="61"/>
+      <c r="E355" s="63"/>
     </row>
     <row r="356" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A356" s="10"/>
       <c r="B356" s="17"/>
       <c r="C356" s="18"/>
       <c r="D356" s="13"/>
-      <c r="E356" s="61"/>
+      <c r="E356" s="63"/>
     </row>
     <row r="357" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A357" s="10"/>
       <c r="B357" s="17"/>
       <c r="C357" s="18"/>
       <c r="D357" s="13"/>
-      <c r="E357" s="61"/>
+      <c r="E357" s="63"/>
     </row>
     <row r="358" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A358" s="10"/>
@@ -6231,14 +6216,14 @@
       <c r="D358" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="E358" s="61"/>
+      <c r="E358" s="63"/>
     </row>
     <row r="359" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A359" s="10"/>
       <c r="B359" s="19"/>
       <c r="C359" s="18"/>
       <c r="D359" s="13"/>
-      <c r="E359" s="61"/>
+      <c r="E359" s="63"/>
     </row>
     <row r="360" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A360" s="10"/>
@@ -6249,7 +6234,7 @@
       <c r="D360" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="E360" s="61"/>
+      <c r="E360" s="63"/>
     </row>
     <row r="361" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A361" s="21" t="s">
@@ -6262,14 +6247,14 @@
       <c r="D361" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="E361" s="61"/>
+      <c r="E361" s="63"/>
     </row>
     <row r="362" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A362" s="10"/>
       <c r="B362" s="10"/>
       <c r="C362" s="10"/>
       <c r="D362" s="13"/>
-      <c r="E362" s="61"/>
+      <c r="E362" s="63"/>
     </row>
     <row r="363" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A363" s="10"/>
@@ -6280,7 +6265,7 @@
       <c r="D363" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="E363" s="61"/>
+      <c r="E363" s="63"/>
     </row>
     <row r="364" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A364" s="10"/>
@@ -6293,7 +6278,7 @@
       <c r="D364" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="E364" s="61"/>
+      <c r="E364" s="63"/>
     </row>
     <row r="365" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A365" s="10"/>
@@ -6306,7 +6291,7 @@
       <c r="D365" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="E365" s="61"/>
+      <c r="E365" s="63"/>
     </row>
     <row r="366" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A366" s="10"/>
@@ -6317,7 +6302,7 @@
       <c r="D366" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="E366" s="61"/>
+      <c r="E366" s="63"/>
     </row>
     <row r="367" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A367" s="28"/>
@@ -6328,7 +6313,7 @@
       <c r="D367" s="30" t="s">
         <v>216</v>
       </c>
-      <c r="E367" s="62"/>
+      <c r="E367" s="64"/>
     </row>
     <row r="368" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A368" s="10"/>
@@ -6343,7 +6328,7 @@
       <c r="B369" s="10"/>
       <c r="C369" s="10"/>
       <c r="D369" s="11"/>
-      <c r="E369" s="61" t="s">
+      <c r="E369" s="63" t="s">
         <v>218</v>
       </c>
     </row>
@@ -6352,7 +6337,7 @@
       <c r="B370" s="10"/>
       <c r="C370" s="10"/>
       <c r="D370" s="13"/>
-      <c r="E370" s="61"/>
+      <c r="E370" s="63"/>
     </row>
     <row r="371" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A371" s="10" t="s">
@@ -6363,7 +6348,7 @@
       </c>
       <c r="C371" s="17"/>
       <c r="D371" s="13"/>
-      <c r="E371" s="61"/>
+      <c r="E371" s="63"/>
     </row>
     <row r="372" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A372" s="10"/>
@@ -6374,7 +6359,7 @@
       <c r="D372" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="E372" s="61"/>
+      <c r="E372" s="63"/>
     </row>
     <row r="373" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A373" s="10"/>
@@ -6385,7 +6370,7 @@
       <c r="D373" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="E373" s="61"/>
+      <c r="E373" s="63"/>
     </row>
     <row r="374" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A374" s="10"/>
@@ -6396,7 +6381,7 @@
       <c r="D374" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="E374" s="61"/>
+      <c r="E374" s="63"/>
     </row>
     <row r="375" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A375" s="10"/>
@@ -6407,7 +6392,7 @@
       <c r="D375" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="E375" s="61"/>
+      <c r="E375" s="63"/>
     </row>
     <row r="376" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A376" s="10"/>
@@ -6418,7 +6403,7 @@
       <c r="D376" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="E376" s="61"/>
+      <c r="E376" s="63"/>
     </row>
     <row r="377" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A377" s="10"/>
@@ -6429,14 +6414,14 @@
       <c r="D377" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="E377" s="61"/>
+      <c r="E377" s="63"/>
     </row>
     <row r="378" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A378" s="10"/>
       <c r="B378" s="44"/>
       <c r="C378" s="17"/>
       <c r="D378" s="13"/>
-      <c r="E378" s="61"/>
+      <c r="E378" s="63"/>
     </row>
     <row r="379" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A379" s="10" t="s">
@@ -6447,7 +6432,7 @@
       </c>
       <c r="C379" s="17"/>
       <c r="D379" s="13"/>
-      <c r="E379" s="61"/>
+      <c r="E379" s="63"/>
     </row>
     <row r="380" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A380" s="10"/>
@@ -6458,7 +6443,7 @@
       <c r="D380" s="13" t="s">
         <v>235</v>
       </c>
-      <c r="E380" s="61"/>
+      <c r="E380" s="63"/>
     </row>
     <row r="381" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A381" s="10"/>
@@ -6469,7 +6454,7 @@
       <c r="D381" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="E381" s="61"/>
+      <c r="E381" s="63"/>
     </row>
     <row r="382" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A382" s="10"/>
@@ -6480,7 +6465,7 @@
       <c r="D382" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="E382" s="61"/>
+      <c r="E382" s="63"/>
     </row>
     <row r="383" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A383" s="10"/>
@@ -6491,7 +6476,7 @@
       <c r="D383" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="E383" s="61"/>
+      <c r="E383" s="63"/>
     </row>
     <row r="384" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A384" s="10"/>
@@ -6502,7 +6487,7 @@
       <c r="D384" s="13" t="s">
         <v>239</v>
       </c>
-      <c r="E384" s="61"/>
+      <c r="E384" s="63"/>
     </row>
     <row r="385" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A385" s="10"/>
@@ -6513,34 +6498,34 @@
       <c r="D385" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="E385" s="61"/>
+      <c r="E385" s="63"/>
     </row>
     <row r="386" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A386" s="10"/>
       <c r="B386" s="44"/>
       <c r="C386" s="18"/>
       <c r="D386" s="13"/>
-      <c r="E386" s="61"/>
+      <c r="E386" s="63"/>
     </row>
     <row r="387" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A387" s="31"/>
       <c r="B387" s="48"/>
       <c r="C387" s="49"/>
       <c r="D387" s="32"/>
-      <c r="E387" s="61"/>
+      <c r="E387" s="63"/>
     </row>
     <row r="388" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A388" s="23" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B388" s="17"/>
       <c r="C388" s="18"/>
       <c r="D388" s="13"/>
-      <c r="E388" s="61"/>
+      <c r="E388" s="63"/>
     </row>
     <row r="389" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A389" s="23" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B389" s="17" t="s">
         <v>241</v>
@@ -6549,11 +6534,11 @@
       <c r="D389" s="13" t="s">
         <v>242</v>
       </c>
-      <c r="E389" s="61"/>
+      <c r="E389" s="63"/>
     </row>
     <row r="390" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A390" s="23" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B390" s="17" t="s">
         <v>243</v>
@@ -6562,11 +6547,11 @@
       <c r="D390" s="13" t="s">
         <v>244</v>
       </c>
-      <c r="E390" s="61"/>
+      <c r="E390" s="63"/>
     </row>
     <row r="391" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A391" s="23" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B391" s="17"/>
       <c r="C391" s="18" t="s">
@@ -6575,29 +6560,29 @@
       <c r="D391" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="E391" s="61"/>
+      <c r="E391" s="63"/>
     </row>
     <row r="392" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A392" s="23" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="B392" s="17"/>
       <c r="C392" s="20"/>
       <c r="D392" s="13"/>
-      <c r="E392" s="61"/>
+      <c r="E392" s="63"/>
     </row>
     <row r="393" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A393" s="23" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="B393" s="10"/>
       <c r="C393" s="10"/>
       <c r="D393" s="13"/>
-      <c r="E393" s="61"/>
+      <c r="E393" s="63"/>
     </row>
     <row r="394" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A394" s="23" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B394" s="26" t="s">
         <v>32</v>
@@ -6606,7 +6591,7 @@
       <c r="D394" s="27" t="s">
         <v>247</v>
       </c>
-      <c r="E394" s="61"/>
+      <c r="E394" s="63"/>
     </row>
     <row r="395" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B395" s="9" t="s">
@@ -6618,7 +6603,7 @@
       <c r="D395" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="E395" s="61"/>
+      <c r="E395" s="63"/>
     </row>
     <row r="396" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A396" s="23"/>
@@ -6631,7 +6616,7 @@
       <c r="D396" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="E396" s="61"/>
+      <c r="E396" s="63"/>
     </row>
     <row r="397" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A397" s="10"/>
@@ -6642,7 +6627,7 @@
       <c r="D397" s="13" t="s">
         <v>250</v>
       </c>
-      <c r="E397" s="61"/>
+      <c r="E397" s="63"/>
     </row>
     <row r="398" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A398" s="28"/>
@@ -6653,7 +6638,7 @@
       <c r="D398" s="30" t="s">
         <v>251</v>
       </c>
-      <c r="E398" s="62"/>
+      <c r="E398" s="64"/>
     </row>
     <row r="399" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A399" s="10"/>
@@ -6668,7 +6653,7 @@
       <c r="B400" s="9"/>
       <c r="C400" s="10"/>
       <c r="D400" s="13"/>
-      <c r="E400" s="61" t="s">
+      <c r="E400" s="63" t="s">
         <v>253</v>
       </c>
     </row>
@@ -6679,7 +6664,7 @@
       <c r="B401" s="9"/>
       <c r="C401" s="10"/>
       <c r="D401" s="50"/>
-      <c r="E401" s="61"/>
+      <c r="E401" s="63"/>
     </row>
     <row r="402" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A402" s="15" t="s">
@@ -6688,7 +6673,7 @@
       <c r="B402" s="23"/>
       <c r="C402" s="10"/>
       <c r="D402" s="33"/>
-      <c r="E402" s="61"/>
+      <c r="E402" s="63"/>
     </row>
     <row r="403" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A403" s="51" t="s">
@@ -6697,27 +6682,27 @@
       <c r="B403" s="17" t="s">
         <v>257</v>
       </c>
-      <c r="C403" s="74" t="s">
+      <c r="C403" s="59" t="s">
         <v>258</v>
       </c>
       <c r="D403" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="E403" s="61"/>
+      <c r="E403" s="63"/>
     </row>
     <row r="404" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A404" s="15"/>
       <c r="B404" s="17"/>
       <c r="C404" s="52"/>
       <c r="D404" s="13"/>
-      <c r="E404" s="61"/>
+      <c r="E404" s="63"/>
     </row>
     <row r="405" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A405" s="15"/>
       <c r="B405" s="10"/>
       <c r="C405" s="10"/>
       <c r="D405" s="13"/>
-      <c r="E405" s="61"/>
+      <c r="E405" s="63"/>
     </row>
     <row r="406" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A406" s="21"/>
@@ -6728,7 +6713,7 @@
       <c r="D406" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="E406" s="61"/>
+      <c r="E406" s="63"/>
     </row>
     <row r="407" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A407" s="10"/>
@@ -6741,7 +6726,7 @@
       <c r="D407" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="E407" s="61"/>
+      <c r="E407" s="63"/>
     </row>
     <row r="408" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A408" s="10"/>
@@ -6754,14 +6739,14 @@
       <c r="D408" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="E408" s="61"/>
+      <c r="E408" s="63"/>
     </row>
     <row r="409" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A409" s="10"/>
       <c r="B409" s="9"/>
       <c r="C409" s="10"/>
       <c r="D409" s="13"/>
-      <c r="E409" s="61"/>
+      <c r="E409" s="63"/>
     </row>
     <row r="410" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A410" s="28"/>
@@ -6770,9 +6755,9 @@
       </c>
       <c r="C410" s="28"/>
       <c r="D410" s="30" t="s">
-        <v>264</v>
-      </c>
-      <c r="E410" s="62"/>
+        <v>263</v>
+      </c>
+      <c r="E410" s="64"/>
     </row>
     <row r="411" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A411" s="10"/>
@@ -6782,13 +6767,13 @@
     </row>
     <row r="412" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A412" s="9" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B412" s="10"/>
       <c r="C412" s="10"/>
       <c r="D412" s="13"/>
-      <c r="E412" s="61" t="s">
-        <v>266</v>
+      <c r="E412" s="63" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="413" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
@@ -6796,115 +6781,115 @@
       <c r="B413" s="10"/>
       <c r="C413" s="10"/>
       <c r="D413" s="13"/>
-      <c r="E413" s="61"/>
+      <c r="E413" s="63"/>
     </row>
     <row r="414" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A414" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B414" s="10"/>
       <c r="C414" s="10"/>
       <c r="D414" s="13"/>
-      <c r="E414" s="61"/>
+      <c r="E414" s="63"/>
     </row>
     <row r="415" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A415" s="10"/>
       <c r="B415" s="10"/>
       <c r="C415" s="10"/>
       <c r="D415" s="13"/>
-      <c r="E415" s="61"/>
+      <c r="E415" s="63"/>
     </row>
     <row r="416" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A416" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="B416" s="13" t="s">
         <v>268</v>
       </c>
-      <c r="B416" s="13" t="s">
+      <c r="C416" s="59" t="s">
         <v>269</v>
       </c>
-      <c r="C416" s="76" t="s">
+      <c r="D416" s="13" t="s">
         <v>270</v>
       </c>
-      <c r="D416" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="E416" s="61"/>
+      <c r="E416" s="63"/>
     </row>
     <row r="417" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A417" s="10"/>
       <c r="B417" s="13"/>
       <c r="C417" s="34"/>
       <c r="D417" s="13"/>
-      <c r="E417" s="61"/>
+      <c r="E417" s="63"/>
     </row>
     <row r="418" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A418" s="10"/>
       <c r="B418" s="13"/>
       <c r="C418" s="34"/>
       <c r="D418" s="13"/>
-      <c r="E418" s="61"/>
+      <c r="E418" s="63"/>
     </row>
     <row r="419" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A419" s="10"/>
       <c r="B419" s="13"/>
       <c r="C419" s="34"/>
       <c r="D419" s="13"/>
-      <c r="E419" s="61"/>
+      <c r="E419" s="63"/>
     </row>
     <row r="420" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A420" s="10"/>
       <c r="B420" s="13"/>
       <c r="C420" s="34"/>
       <c r="D420" s="13"/>
-      <c r="E420" s="61"/>
+      <c r="E420" s="63"/>
     </row>
     <row r="421" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A421" s="10"/>
       <c r="B421" s="13"/>
       <c r="C421" s="34"/>
       <c r="D421" s="13"/>
-      <c r="E421" s="61"/>
+      <c r="E421" s="63"/>
     </row>
     <row r="422" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A422" s="10"/>
       <c r="B422" s="13"/>
       <c r="C422" s="34"/>
       <c r="D422" s="13"/>
-      <c r="E422" s="61"/>
+      <c r="E422" s="63"/>
     </row>
     <row r="423" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A423" s="10"/>
       <c r="B423" s="13"/>
       <c r="C423" s="10"/>
       <c r="D423" s="13"/>
-      <c r="E423" s="61"/>
+      <c r="E423" s="63"/>
     </row>
     <row r="424" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A424" s="10"/>
       <c r="B424" s="13"/>
       <c r="C424" s="10"/>
       <c r="D424" s="13"/>
-      <c r="E424" s="61"/>
+      <c r="E424" s="63"/>
     </row>
     <row r="425" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A425" s="10"/>
       <c r="B425" s="10"/>
       <c r="C425" s="10"/>
       <c r="D425" s="33"/>
-      <c r="E425" s="61"/>
+      <c r="E425" s="63"/>
     </row>
     <row r="426" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A426" s="9"/>
       <c r="B426" s="17"/>
       <c r="C426" s="34"/>
       <c r="D426" s="13"/>
-      <c r="E426" s="61"/>
+      <c r="E426" s="63"/>
     </row>
     <row r="427" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A427" s="10"/>
       <c r="B427" s="10"/>
       <c r="C427" s="10"/>
       <c r="D427" s="13"/>
-      <c r="E427" s="61"/>
+      <c r="E427" s="63"/>
     </row>
     <row r="428" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A428" s="21"/>
@@ -6913,9 +6898,9 @@
       </c>
       <c r="C428" s="10"/>
       <c r="D428" s="13" t="s">
-        <v>272</v>
-      </c>
-      <c r="E428" s="61"/>
+        <v>271</v>
+      </c>
+      <c r="E428" s="63"/>
     </row>
     <row r="429" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A429" s="10"/>
@@ -6926,9 +6911,9 @@
         <v>2.5000000000000001E-3</v>
       </c>
       <c r="D429" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="E429" s="61"/>
+        <v>272</v>
+      </c>
+      <c r="E429" s="63"/>
     </row>
     <row r="430" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A430" s="10"/>
@@ -6939,23 +6924,23 @@
         <v>2E-3</v>
       </c>
       <c r="D430" s="13" t="s">
-        <v>274</v>
-      </c>
-      <c r="E430" s="61"/>
+        <v>273</v>
+      </c>
+      <c r="E430" s="63"/>
     </row>
     <row r="431" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A431" s="10"/>
       <c r="B431" s="9"/>
       <c r="C431" s="10"/>
       <c r="D431" s="13"/>
-      <c r="E431" s="61"/>
+      <c r="E431" s="63"/>
     </row>
     <row r="432" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A432" s="10"/>
       <c r="B432" s="9"/>
       <c r="C432" s="10"/>
       <c r="D432" s="13"/>
-      <c r="E432" s="61"/>
+      <c r="E432" s="63"/>
     </row>
     <row r="433" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A433" s="28"/>
@@ -6964,9 +6949,9 @@
       </c>
       <c r="C433" s="28"/>
       <c r="D433" s="30" t="s">
-        <v>276</v>
-      </c>
-      <c r="E433" s="62"/>
+        <v>274</v>
+      </c>
+      <c r="E433" s="64"/>
     </row>
     <row r="434" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A434" s="10"/>
@@ -6976,13 +6961,13 @@
     </row>
     <row r="435" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A435" s="9" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B435" s="10"/>
       <c r="C435" s="10"/>
       <c r="D435" s="13"/>
-      <c r="E435" s="61" t="s">
-        <v>266</v>
+      <c r="E435" s="63" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="436" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
@@ -6990,101 +6975,101 @@
       <c r="B436" s="10"/>
       <c r="C436" s="10"/>
       <c r="D436" s="13"/>
-      <c r="E436" s="61"/>
+      <c r="E436" s="63"/>
     </row>
     <row r="437" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A437" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B437" s="13"/>
       <c r="C437" s="34"/>
       <c r="D437" s="13"/>
-      <c r="E437" s="61"/>
+      <c r="E437" s="63"/>
     </row>
     <row r="438" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A438" s="10"/>
       <c r="B438" s="13"/>
       <c r="C438" s="34"/>
       <c r="D438" s="13"/>
-      <c r="E438" s="61"/>
+      <c r="E438" s="63"/>
     </row>
     <row r="439" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A439" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="B439" s="13" t="s">
         <v>268</v>
       </c>
-      <c r="B439" s="13" t="s">
+      <c r="C439" s="59" t="s">
         <v>269</v>
       </c>
-      <c r="C439" s="76" t="s">
+      <c r="D439" s="13" t="s">
         <v>270</v>
       </c>
-      <c r="D439" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="E439" s="61"/>
+      <c r="E439" s="63"/>
     </row>
     <row r="440" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A440" s="10"/>
       <c r="B440" s="13"/>
       <c r="C440" s="34"/>
       <c r="D440" s="13"/>
-      <c r="E440" s="61"/>
+      <c r="E440" s="63"/>
     </row>
     <row r="441" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A441" s="10"/>
       <c r="B441" s="13"/>
       <c r="C441" s="34"/>
       <c r="D441" s="13"/>
-      <c r="E441" s="61"/>
+      <c r="E441" s="63"/>
     </row>
     <row r="442" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A442" s="10"/>
       <c r="B442" s="13"/>
       <c r="C442" s="34"/>
       <c r="D442" s="13"/>
-      <c r="E442" s="61"/>
+      <c r="E442" s="63"/>
     </row>
     <row r="443" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A443" s="10"/>
       <c r="B443" s="13"/>
       <c r="C443" s="34"/>
       <c r="D443" s="13"/>
-      <c r="E443" s="61"/>
+      <c r="E443" s="63"/>
     </row>
     <row r="444" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A444" s="10"/>
       <c r="B444" s="13"/>
       <c r="C444" s="10"/>
       <c r="D444" s="13"/>
-      <c r="E444" s="61"/>
+      <c r="E444" s="63"/>
     </row>
     <row r="445" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A445" s="10"/>
       <c r="B445" s="13"/>
       <c r="C445" s="10"/>
       <c r="D445" s="13"/>
-      <c r="E445" s="61"/>
+      <c r="E445" s="63"/>
     </row>
     <row r="446" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A446" s="10"/>
       <c r="B446" s="10"/>
       <c r="C446" s="10"/>
       <c r="D446" s="33"/>
-      <c r="E446" s="61"/>
+      <c r="E446" s="63"/>
     </row>
     <row r="447" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A447" s="9"/>
       <c r="B447" s="17"/>
       <c r="C447" s="34"/>
       <c r="D447" s="13"/>
-      <c r="E447" s="61"/>
+      <c r="E447" s="63"/>
     </row>
     <row r="448" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A448" s="10"/>
       <c r="B448" s="10"/>
       <c r="C448" s="10"/>
       <c r="D448" s="13"/>
-      <c r="E448" s="61"/>
+      <c r="E448" s="63"/>
     </row>
     <row r="449" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A449" s="21"/>
@@ -7093,9 +7078,9 @@
       </c>
       <c r="C449" s="10"/>
       <c r="D449" s="13" t="s">
-        <v>272</v>
-      </c>
-      <c r="E449" s="61"/>
+        <v>271</v>
+      </c>
+      <c r="E449" s="63"/>
     </row>
     <row r="450" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A450" s="10"/>
@@ -7106,9 +7091,9 @@
         <v>2.5000000000000001E-3</v>
       </c>
       <c r="D450" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="E450" s="61"/>
+        <v>272</v>
+      </c>
+      <c r="E450" s="63"/>
     </row>
     <row r="451" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A451" s="10"/>
@@ -7119,23 +7104,23 @@
         <v>2E-3</v>
       </c>
       <c r="D451" s="13" t="s">
-        <v>274</v>
-      </c>
-      <c r="E451" s="61"/>
+        <v>273</v>
+      </c>
+      <c r="E451" s="63"/>
     </row>
     <row r="452" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A452" s="10"/>
       <c r="B452" s="9"/>
       <c r="C452" s="10"/>
       <c r="D452" s="13"/>
-      <c r="E452" s="61"/>
+      <c r="E452" s="63"/>
     </row>
     <row r="453" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A453" s="10"/>
       <c r="B453" s="9"/>
       <c r="C453" s="10"/>
       <c r="D453" s="13"/>
-      <c r="E453" s="61"/>
+      <c r="E453" s="63"/>
     </row>
     <row r="454" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A454" s="28"/>
@@ -7144,9 +7129,9 @@
       </c>
       <c r="C454" s="28"/>
       <c r="D454" s="30" t="s">
-        <v>276</v>
-      </c>
-      <c r="E454" s="62"/>
+        <v>274</v>
+      </c>
+      <c r="E454" s="64"/>
     </row>
     <row r="455" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A455" s="9"/>
@@ -7156,13 +7141,13 @@
     </row>
     <row r="456" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A456" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B456" s="10"/>
       <c r="C456" s="10"/>
       <c r="D456" s="13"/>
-      <c r="E456" s="60" t="s">
-        <v>279</v>
+      <c r="E456" s="62" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="457" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
@@ -7170,101 +7155,101 @@
       <c r="B457" s="10"/>
       <c r="C457" s="10"/>
       <c r="D457" s="13"/>
-      <c r="E457" s="61"/>
+      <c r="E457" s="63"/>
     </row>
     <row r="458" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A458" s="10" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B458" s="13"/>
       <c r="C458" s="34"/>
       <c r="D458" s="13"/>
-      <c r="E458" s="61"/>
+      <c r="E458" s="63"/>
     </row>
     <row r="459" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A459" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="B459" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="C459" s="59" t="s">
         <v>281</v>
       </c>
-      <c r="B459" s="13" t="s">
+      <c r="D459" s="13" t="s">
         <v>282</v>
       </c>
-      <c r="C459" s="76" t="s">
-        <v>283</v>
-      </c>
-      <c r="D459" s="13" t="s">
-        <v>284</v>
-      </c>
-      <c r="E459" s="61"/>
+      <c r="E459" s="63"/>
     </row>
     <row r="460" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A460" s="10"/>
       <c r="B460" s="13"/>
       <c r="C460" s="34"/>
       <c r="D460" s="13"/>
-      <c r="E460" s="61"/>
+      <c r="E460" s="63"/>
     </row>
     <row r="461" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A461" s="10"/>
       <c r="B461" s="13"/>
       <c r="C461" s="34"/>
       <c r="D461" s="13"/>
-      <c r="E461" s="61"/>
+      <c r="E461" s="63"/>
     </row>
     <row r="462" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A462" s="10"/>
       <c r="B462" s="13"/>
       <c r="C462" s="34"/>
       <c r="D462" s="13"/>
-      <c r="E462" s="61"/>
+      <c r="E462" s="63"/>
     </row>
     <row r="463" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A463" s="10"/>
       <c r="B463" s="13"/>
       <c r="C463" s="34"/>
       <c r="D463" s="13"/>
-      <c r="E463" s="61"/>
+      <c r="E463" s="63"/>
     </row>
     <row r="464" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A464" s="10"/>
       <c r="B464" s="13"/>
       <c r="C464" s="34"/>
       <c r="D464" s="13"/>
-      <c r="E464" s="61"/>
+      <c r="E464" s="63"/>
     </row>
     <row r="465" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A465" s="10"/>
       <c r="B465" s="13"/>
       <c r="C465" s="10"/>
       <c r="D465" s="13"/>
-      <c r="E465" s="61"/>
+      <c r="E465" s="63"/>
     </row>
     <row r="466" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A466" s="10"/>
       <c r="B466" s="13"/>
       <c r="C466" s="10"/>
       <c r="D466" s="13"/>
-      <c r="E466" s="61"/>
+      <c r="E466" s="63"/>
     </row>
     <row r="467" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A467" s="10"/>
       <c r="B467" s="10"/>
       <c r="C467" s="10"/>
       <c r="D467" s="33"/>
-      <c r="E467" s="61"/>
+      <c r="E467" s="63"/>
     </row>
     <row r="468" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A468" s="9"/>
       <c r="B468" s="17"/>
       <c r="C468" s="34"/>
       <c r="D468" s="13"/>
-      <c r="E468" s="61"/>
+      <c r="E468" s="63"/>
     </row>
     <row r="469" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A469" s="10"/>
       <c r="B469" s="10"/>
       <c r="C469" s="10"/>
       <c r="D469" s="13"/>
-      <c r="E469" s="61"/>
+      <c r="E469" s="63"/>
     </row>
     <row r="470" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A470" s="21"/>
@@ -7273,9 +7258,9 @@
       </c>
       <c r="C470" s="10"/>
       <c r="D470" s="13" t="s">
-        <v>285</v>
-      </c>
-      <c r="E470" s="61"/>
+        <v>283</v>
+      </c>
+      <c r="E470" s="63"/>
     </row>
     <row r="471" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A471" s="10"/>
@@ -7286,9 +7271,9 @@
         <v>2.5000000000000001E-3</v>
       </c>
       <c r="D471" s="13" t="s">
-        <v>286</v>
-      </c>
-      <c r="E471" s="61"/>
+        <v>284</v>
+      </c>
+      <c r="E471" s="63"/>
     </row>
     <row r="472" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A472" s="10"/>
@@ -7299,16 +7284,16 @@
         <v>2E-3</v>
       </c>
       <c r="D472" s="13" t="s">
-        <v>287</v>
-      </c>
-      <c r="E472" s="61"/>
+        <v>285</v>
+      </c>
+      <c r="E472" s="63"/>
     </row>
     <row r="473" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A473" s="10"/>
       <c r="B473" s="9"/>
       <c r="C473" s="10"/>
       <c r="D473" s="13"/>
-      <c r="E473" s="61"/>
+      <c r="E473" s="63"/>
     </row>
     <row r="474" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A474" s="28"/>
@@ -7317,26 +7302,26 @@
       </c>
       <c r="C474" s="28"/>
       <c r="D474" s="30" t="s">
-        <v>289</v>
-      </c>
-      <c r="E474" s="62"/>
+        <v>286</v>
+      </c>
+      <c r="E474" s="64"/>
     </row>
     <row r="475" spans="1:5" ht="15.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A475" s="63"/>
-      <c r="B475" s="65" t="s">
-        <v>290</v>
+      <c r="A475" s="65"/>
+      <c r="B475" s="67" t="s">
+        <v>287</v>
       </c>
       <c r="C475" s="53"/>
-      <c r="D475" s="67" t="s">
-        <v>291</v>
+      <c r="D475" s="69" t="s">
+        <v>288</v>
       </c>
       <c r="E475" s="54"/>
     </row>
     <row r="476" spans="1:5" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A476" s="64"/>
-      <c r="B476" s="66"/>
+      <c r="A476" s="66"/>
+      <c r="B476" s="68"/>
       <c r="C476" s="55"/>
-      <c r="D476" s="68"/>
+      <c r="D476" s="70"/>
       <c r="E476" s="56"/>
     </row>
   </sheetData>

</xml_diff>